<commit_message>
Integrate RFQ v32 and simplify guided automation workflows
</commit_message>
<xml_diff>
--- a/resources/templates/Create_RFQ_Template.xlsx
+++ b/resources/templates/Create_RFQ_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RPA_Input" sheetId="1" r:id="R9cab2fe0865647d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R6aa974072bd04dd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RPA_Input" sheetId="1" r:id="R168a6f4efe2643aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rbee507f2be4f4876"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -119,9 +119,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="202" formatCode="0.########"/>
+    <x:numFmt numFmtId="203" formatCode="General"/>
   </x:numFmts>
   <x:fonts count="9">
     <x:font>
@@ -175,7 +177,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -222,8 +224,48 @@
         <x:fgColor rgb="FFFFF2F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF506477"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF506477"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF245E98"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF9E9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF245E98"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF9E9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="6">
+  <x:borders count="7">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -295,11 +337,25 @@
         <x:color rgb="FFE9B7BC"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFDAE3F0"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFDAE3F0"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFDAE3F0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFDAE3F0"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="77">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -385,33 +441,166 @@
     <x:xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="17" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="17" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="17" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
+  <x:dxfs count="4">
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FFB91C1C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FFB91C1C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FFB91C1C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FFB91C1C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
   <xltc:person displayName="SAP Automation Toolbox" id="{459AB45E-2731-4CC1-958B-F9AA8585CA2B}"/>
+  <xltc:person displayName="User" id="{A2EAAE16-A3FC-4C51-82EF-9E9215AB87B8}"/>
 </xltc:personList>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CreateRfqInput" displayName="CreateRfqInput" ref="A1:H201" headerRowCount="1">
-  <x:autoFilter ref="A1:H201"/>
-  <x:tableColumns count="8">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CreateRfqInput" displayName="CreateRfqInput" ref="A1:L201" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:L201"/>
+  <x:tableColumns count="12">
     <x:tableColumn id="1" name="Plant"/>
     <x:tableColumn id="2" name="Project No."/>
     <x:tableColumn id="3" name="Material No."/>
-    <x:tableColumn id="4" name="Intended Supplier"/>
+    <x:tableColumn id="4" name="Supplier Parma"/>
     <x:tableColumn id="5" name="Supplier Email"/>
     <x:tableColumn id="6" name="Quotation Due Date"/>
     <x:tableColumn id="7" name="PPAP Date"/>
     <x:tableColumn id="8" name="Technology"/>
+    <x:tableColumn id="9" name="12 MR Qty"/>
+    <x:tableColumn id="10" name="RFQ Qty Prototype"/>
+    <x:tableColumn id="11" name="RFQ Qty Serial"/>
+    <x:tableColumn id="12" name="Cost Breakdown"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -458,9 +647,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -590,9 +779,17 @@
     <xltc:text>可选。Buyer Receipt 中 PPAP 日期为空或已过期时使用；格式 YYYY-MM-DD。
 Optional fallback PPAP date in YYYY-MM-DD format.</xltc:text>
   </xltc:threadedComment>
+  <xltc:threadedComment ref="G1" dT="2026-09-30T07:08:22.105" personId="{A2EAAE16-A3FC-4C51-82EF-9E9215AB87B8}" id="{66728191-AF48-491B-A2EF-FF723D1CBAC7}" parentId="{B194F078-DBFE-541F-5E97-8B6B59E7C0C5}">
+    <xltc:text>更新：G 列 PPAP Date 现为必填，不再是选填。日期格式 YYYY-MM-DD。
+Updated: PPAP Date is required. Use YYYY-MM-DD.</xltc:text>
+  </xltc:threadedComment>
   <xltc:threadedComment ref="H1" dT="2026-08-07T06:43:21.778" personId="{459AB45E-2731-4CC1-958B-F9AA8585CA2B}" id="{9FA00706-1438-4768-B01E-B76E9745E30B}">
     <xltc:text>可选。负责该物料的 Technology User。
 Optional Technology User for the material.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="H1" dT="2026-09-30T07:08:22.109" personId="{A2EAAE16-A3FC-4C51-82EF-9E9215AB87B8}" id="{D107BD72-36BE-48D2-B3E3-01E9FD04816A}" parentId="{9FA00706-1438-4768-B01E-B76E9745E30B}">
+    <xltc:text>更新：H 列 Technology 现为必填，不再是选填。填写负责该物料的技术负责人。
+Updated: Technology is required. Enter the Technology User for this material.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
 </file>
@@ -609,6 +806,10 @@
     <x:col min="6" max="6" width="21" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="21" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="23" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="23" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="23" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
@@ -622,7 +823,7 @@
         <x:v>Material No.</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>Intended Supplier</x:v>
+        <x:v>Supplier Parma</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
         <x:v>Supplier Email</x:v>
@@ -630,11 +831,23 @@
       <x:c r="F1" s="6" t="str">
         <x:v>Quotation Due Date</x:v>
       </x:c>
-      <x:c r="G1" s="12" t="str">
+      <x:c r="G1" s="72" t="str">
         <x:v>PPAP Date</x:v>
       </x:c>
-      <x:c r="H1" s="12" t="str">
+      <x:c r="H1" s="72" t="str">
         <x:v>Technology</x:v>
+      </x:c>
+      <x:c r="I1" s="75" t="str">
+        <x:v>12 MR Qty</x:v>
+      </x:c>
+      <x:c r="J1" s="63" t="str">
+        <x:v>RFQ Qty Prototype</x:v>
+      </x:c>
+      <x:c r="K1" s="75" t="str">
+        <x:v>RFQ Qty Serial</x:v>
+      </x:c>
+      <x:c r="L1" s="63" t="str">
+        <x:v>Cost Breakdown</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
@@ -646,8 +859,14 @@
       <x:c r="D2" s="21"/>
       <x:c r="E2" s="21"/>
       <x:c r="F2" s="22"/>
-      <x:c r="G2" s="23"/>
-      <x:c r="H2" s="24"/>
+      <x:c r="G2" s="73"/>
+      <x:c r="H2" s="74"/>
+      <x:c r="I2" s="76"/>
+      <x:c r="J2" s="64"/>
+      <x:c r="K2" s="76"/>
+      <x:c r="L2" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="21" t="str">
@@ -658,8 +877,14 @@
       <x:c r="D3" s="21"/>
       <x:c r="E3" s="21"/>
       <x:c r="F3" s="22"/>
-      <x:c r="G3" s="23"/>
-      <x:c r="H3" s="24"/>
+      <x:c r="G3" s="73"/>
+      <x:c r="H3" s="74"/>
+      <x:c r="I3" s="76"/>
+      <x:c r="J3" s="64"/>
+      <x:c r="K3" s="76"/>
+      <x:c r="L3" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="21" t="str">
@@ -670,8 +895,14 @@
       <x:c r="D4" s="21"/>
       <x:c r="E4" s="21"/>
       <x:c r="F4" s="22"/>
-      <x:c r="G4" s="23"/>
-      <x:c r="H4" s="24"/>
+      <x:c r="G4" s="73"/>
+      <x:c r="H4" s="74"/>
+      <x:c r="I4" s="76"/>
+      <x:c r="J4" s="64"/>
+      <x:c r="K4" s="76"/>
+      <x:c r="L4" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="A5" s="21" t="str">
@@ -682,8 +913,14 @@
       <x:c r="D5" s="21"/>
       <x:c r="E5" s="21"/>
       <x:c r="F5" s="22"/>
-      <x:c r="G5" s="23"/>
-      <x:c r="H5" s="24"/>
+      <x:c r="G5" s="73"/>
+      <x:c r="H5" s="74"/>
+      <x:c r="I5" s="76"/>
+      <x:c r="J5" s="64"/>
+      <x:c r="K5" s="76"/>
+      <x:c r="L5" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="21" t="str">
@@ -694,8 +931,14 @@
       <x:c r="D6" s="21"/>
       <x:c r="E6" s="21"/>
       <x:c r="F6" s="22"/>
-      <x:c r="G6" s="23"/>
-      <x:c r="H6" s="24"/>
+      <x:c r="G6" s="73"/>
+      <x:c r="H6" s="74"/>
+      <x:c r="I6" s="76"/>
+      <x:c r="J6" s="64"/>
+      <x:c r="K6" s="76"/>
+      <x:c r="L6" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
       <x:c r="A7" s="21" t="str">
@@ -706,8 +949,14 @@
       <x:c r="D7" s="21"/>
       <x:c r="E7" s="21"/>
       <x:c r="F7" s="22"/>
-      <x:c r="G7" s="23"/>
-      <x:c r="H7" s="24"/>
+      <x:c r="G7" s="73"/>
+      <x:c r="H7" s="74"/>
+      <x:c r="I7" s="76"/>
+      <x:c r="J7" s="64"/>
+      <x:c r="K7" s="76"/>
+      <x:c r="L7" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
       <x:c r="A8" s="21" t="str">
@@ -718,8 +967,14 @@
       <x:c r="D8" s="21"/>
       <x:c r="E8" s="21"/>
       <x:c r="F8" s="22"/>
-      <x:c r="G8" s="23"/>
-      <x:c r="H8" s="24"/>
+      <x:c r="G8" s="73"/>
+      <x:c r="H8" s="74"/>
+      <x:c r="I8" s="76"/>
+      <x:c r="J8" s="64"/>
+      <x:c r="K8" s="76"/>
+      <x:c r="L8" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
       <x:c r="A9" s="21" t="str">
@@ -730,8 +985,14 @@
       <x:c r="D9" s="21"/>
       <x:c r="E9" s="21"/>
       <x:c r="F9" s="22"/>
-      <x:c r="G9" s="23"/>
-      <x:c r="H9" s="24"/>
+      <x:c r="G9" s="73"/>
+      <x:c r="H9" s="74"/>
+      <x:c r="I9" s="76"/>
+      <x:c r="J9" s="64"/>
+      <x:c r="K9" s="76"/>
+      <x:c r="L9" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
       <x:c r="A10" s="21" t="str">
@@ -742,8 +1003,14 @@
       <x:c r="D10" s="21"/>
       <x:c r="E10" s="21"/>
       <x:c r="F10" s="22"/>
-      <x:c r="G10" s="23"/>
-      <x:c r="H10" s="24"/>
+      <x:c r="G10" s="73"/>
+      <x:c r="H10" s="74"/>
+      <x:c r="I10" s="76"/>
+      <x:c r="J10" s="64"/>
+      <x:c r="K10" s="76"/>
+      <x:c r="L10" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
       <x:c r="A11" s="21" t="str">
@@ -754,8 +1021,14 @@
       <x:c r="D11" s="21"/>
       <x:c r="E11" s="21"/>
       <x:c r="F11" s="22"/>
-      <x:c r="G11" s="23"/>
-      <x:c r="H11" s="24"/>
+      <x:c r="G11" s="73"/>
+      <x:c r="H11" s="74"/>
+      <x:c r="I11" s="76"/>
+      <x:c r="J11" s="64"/>
+      <x:c r="K11" s="76"/>
+      <x:c r="L11" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
       <x:c r="A12" s="21" t="str">
@@ -766,8 +1039,14 @@
       <x:c r="D12" s="21"/>
       <x:c r="E12" s="21"/>
       <x:c r="F12" s="22"/>
-      <x:c r="G12" s="23"/>
-      <x:c r="H12" s="24"/>
+      <x:c r="G12" s="73"/>
+      <x:c r="H12" s="74"/>
+      <x:c r="I12" s="76"/>
+      <x:c r="J12" s="64"/>
+      <x:c r="K12" s="76"/>
+      <x:c r="L12" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
       <x:c r="A13" s="21" t="str">
@@ -778,8 +1057,14 @@
       <x:c r="D13" s="21"/>
       <x:c r="E13" s="21"/>
       <x:c r="F13" s="22"/>
-      <x:c r="G13" s="23"/>
-      <x:c r="H13" s="24"/>
+      <x:c r="G13" s="73"/>
+      <x:c r="H13" s="74"/>
+      <x:c r="I13" s="76"/>
+      <x:c r="J13" s="64"/>
+      <x:c r="K13" s="76"/>
+      <x:c r="L13" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
       <x:c r="A14" s="21" t="str">
@@ -790,8 +1075,14 @@
       <x:c r="D14" s="21"/>
       <x:c r="E14" s="21"/>
       <x:c r="F14" s="22"/>
-      <x:c r="G14" s="23"/>
-      <x:c r="H14" s="24"/>
+      <x:c r="G14" s="73"/>
+      <x:c r="H14" s="74"/>
+      <x:c r="I14" s="76"/>
+      <x:c r="J14" s="64"/>
+      <x:c r="K14" s="76"/>
+      <x:c r="L14" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="A15" s="21" t="str">
@@ -802,8 +1093,14 @@
       <x:c r="D15" s="21"/>
       <x:c r="E15" s="21"/>
       <x:c r="F15" s="22"/>
-      <x:c r="G15" s="23"/>
-      <x:c r="H15" s="24"/>
+      <x:c r="G15" s="73"/>
+      <x:c r="H15" s="74"/>
+      <x:c r="I15" s="76"/>
+      <x:c r="J15" s="64"/>
+      <x:c r="K15" s="76"/>
+      <x:c r="L15" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="21" t="str">
@@ -814,8 +1111,14 @@
       <x:c r="D16" s="21"/>
       <x:c r="E16" s="21"/>
       <x:c r="F16" s="22"/>
-      <x:c r="G16" s="23"/>
-      <x:c r="H16" s="24"/>
+      <x:c r="G16" s="73"/>
+      <x:c r="H16" s="74"/>
+      <x:c r="I16" s="76"/>
+      <x:c r="J16" s="64"/>
+      <x:c r="K16" s="76"/>
+      <x:c r="L16" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="21" t="str">
@@ -826,8 +1129,14 @@
       <x:c r="D17" s="21"/>
       <x:c r="E17" s="21"/>
       <x:c r="F17" s="22"/>
-      <x:c r="G17" s="23"/>
-      <x:c r="H17" s="24"/>
+      <x:c r="G17" s="73"/>
+      <x:c r="H17" s="74"/>
+      <x:c r="I17" s="76"/>
+      <x:c r="J17" s="64"/>
+      <x:c r="K17" s="76"/>
+      <x:c r="L17" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="A18" s="21" t="str">
@@ -838,8 +1147,14 @@
       <x:c r="D18" s="21"/>
       <x:c r="E18" s="21"/>
       <x:c r="F18" s="22"/>
-      <x:c r="G18" s="23"/>
-      <x:c r="H18" s="24"/>
+      <x:c r="G18" s="73"/>
+      <x:c r="H18" s="74"/>
+      <x:c r="I18" s="76"/>
+      <x:c r="J18" s="64"/>
+      <x:c r="K18" s="76"/>
+      <x:c r="L18" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19" s="21" t="str">
@@ -850,8 +1165,14 @@
       <x:c r="D19" s="21"/>
       <x:c r="E19" s="21"/>
       <x:c r="F19" s="22"/>
-      <x:c r="G19" s="23"/>
-      <x:c r="H19" s="24"/>
+      <x:c r="G19" s="73"/>
+      <x:c r="H19" s="74"/>
+      <x:c r="I19" s="76"/>
+      <x:c r="J19" s="64"/>
+      <x:c r="K19" s="76"/>
+      <x:c r="L19" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
       <x:c r="A20" s="21" t="str">
@@ -862,8 +1183,14 @@
       <x:c r="D20" s="21"/>
       <x:c r="E20" s="21"/>
       <x:c r="F20" s="22"/>
-      <x:c r="G20" s="23"/>
-      <x:c r="H20" s="24"/>
+      <x:c r="G20" s="73"/>
+      <x:c r="H20" s="74"/>
+      <x:c r="I20" s="76"/>
+      <x:c r="J20" s="64"/>
+      <x:c r="K20" s="76"/>
+      <x:c r="L20" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
       <x:c r="A21" s="21" t="str">
@@ -874,8 +1201,14 @@
       <x:c r="D21" s="21"/>
       <x:c r="E21" s="21"/>
       <x:c r="F21" s="22"/>
-      <x:c r="G21" s="23"/>
-      <x:c r="H21" s="24"/>
+      <x:c r="G21" s="73"/>
+      <x:c r="H21" s="74"/>
+      <x:c r="I21" s="76"/>
+      <x:c r="J21" s="64"/>
+      <x:c r="K21" s="76"/>
+      <x:c r="L21" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="22" customHeight="1">
       <x:c r="A22" s="21" t="str">
@@ -886,8 +1219,14 @@
       <x:c r="D22" s="21"/>
       <x:c r="E22" s="21"/>
       <x:c r="F22" s="22"/>
-      <x:c r="G22" s="23"/>
-      <x:c r="H22" s="24"/>
+      <x:c r="G22" s="73"/>
+      <x:c r="H22" s="74"/>
+      <x:c r="I22" s="76"/>
+      <x:c r="J22" s="64"/>
+      <x:c r="K22" s="76"/>
+      <x:c r="L22" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
       <x:c r="A23" s="21" t="str">
@@ -898,8 +1237,14 @@
       <x:c r="D23" s="21"/>
       <x:c r="E23" s="21"/>
       <x:c r="F23" s="22"/>
-      <x:c r="G23" s="23"/>
-      <x:c r="H23" s="24"/>
+      <x:c r="G23" s="73"/>
+      <x:c r="H23" s="74"/>
+      <x:c r="I23" s="76"/>
+      <x:c r="J23" s="64"/>
+      <x:c r="K23" s="76"/>
+      <x:c r="L23" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
       <x:c r="A24" s="21" t="str">
@@ -910,8 +1255,14 @@
       <x:c r="D24" s="21"/>
       <x:c r="E24" s="21"/>
       <x:c r="F24" s="22"/>
-      <x:c r="G24" s="23"/>
-      <x:c r="H24" s="24"/>
+      <x:c r="G24" s="73"/>
+      <x:c r="H24" s="74"/>
+      <x:c r="I24" s="76"/>
+      <x:c r="J24" s="64"/>
+      <x:c r="K24" s="76"/>
+      <x:c r="L24" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="22" customHeight="1">
       <x:c r="A25" s="21" t="str">
@@ -922,8 +1273,14 @@
       <x:c r="D25" s="21"/>
       <x:c r="E25" s="21"/>
       <x:c r="F25" s="22"/>
-      <x:c r="G25" s="23"/>
-      <x:c r="H25" s="24"/>
+      <x:c r="G25" s="73"/>
+      <x:c r="H25" s="74"/>
+      <x:c r="I25" s="76"/>
+      <x:c r="J25" s="64"/>
+      <x:c r="K25" s="76"/>
+      <x:c r="L25" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="22" customHeight="1">
       <x:c r="A26" s="21" t="str">
@@ -934,8 +1291,14 @@
       <x:c r="D26" s="21"/>
       <x:c r="E26" s="21"/>
       <x:c r="F26" s="22"/>
-      <x:c r="G26" s="23"/>
-      <x:c r="H26" s="24"/>
+      <x:c r="G26" s="73"/>
+      <x:c r="H26" s="74"/>
+      <x:c r="I26" s="76"/>
+      <x:c r="J26" s="64"/>
+      <x:c r="K26" s="76"/>
+      <x:c r="L26" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="22" customHeight="1">
       <x:c r="A27" s="21" t="str">
@@ -946,8 +1309,14 @@
       <x:c r="D27" s="21"/>
       <x:c r="E27" s="21"/>
       <x:c r="F27" s="22"/>
-      <x:c r="G27" s="23"/>
-      <x:c r="H27" s="24"/>
+      <x:c r="G27" s="73"/>
+      <x:c r="H27" s="74"/>
+      <x:c r="I27" s="76"/>
+      <x:c r="J27" s="64"/>
+      <x:c r="K27" s="76"/>
+      <x:c r="L27" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="22" customHeight="1">
       <x:c r="A28" s="21" t="str">
@@ -958,8 +1327,14 @@
       <x:c r="D28" s="21"/>
       <x:c r="E28" s="21"/>
       <x:c r="F28" s="22"/>
-      <x:c r="G28" s="23"/>
-      <x:c r="H28" s="24"/>
+      <x:c r="G28" s="73"/>
+      <x:c r="H28" s="74"/>
+      <x:c r="I28" s="76"/>
+      <x:c r="J28" s="64"/>
+      <x:c r="K28" s="76"/>
+      <x:c r="L28" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="22" customHeight="1">
       <x:c r="A29" s="21" t="str">
@@ -970,8 +1345,14 @@
       <x:c r="D29" s="21"/>
       <x:c r="E29" s="21"/>
       <x:c r="F29" s="22"/>
-      <x:c r="G29" s="23"/>
-      <x:c r="H29" s="24"/>
+      <x:c r="G29" s="73"/>
+      <x:c r="H29" s="74"/>
+      <x:c r="I29" s="76"/>
+      <x:c r="J29" s="64"/>
+      <x:c r="K29" s="76"/>
+      <x:c r="L29" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="22" customHeight="1">
       <x:c r="A30" s="21" t="str">
@@ -982,8 +1363,14 @@
       <x:c r="D30" s="21"/>
       <x:c r="E30" s="21"/>
       <x:c r="F30" s="22"/>
-      <x:c r="G30" s="23"/>
-      <x:c r="H30" s="24"/>
+      <x:c r="G30" s="73"/>
+      <x:c r="H30" s="74"/>
+      <x:c r="I30" s="76"/>
+      <x:c r="J30" s="64"/>
+      <x:c r="K30" s="76"/>
+      <x:c r="L30" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="22" customHeight="1">
       <x:c r="A31" s="21" t="str">
@@ -994,8 +1381,14 @@
       <x:c r="D31" s="21"/>
       <x:c r="E31" s="21"/>
       <x:c r="F31" s="22"/>
-      <x:c r="G31" s="23"/>
-      <x:c r="H31" s="24"/>
+      <x:c r="G31" s="73"/>
+      <x:c r="H31" s="74"/>
+      <x:c r="I31" s="76"/>
+      <x:c r="J31" s="64"/>
+      <x:c r="K31" s="76"/>
+      <x:c r="L31" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="22" customHeight="1">
       <x:c r="A32" s="21" t="str">
@@ -1006,8 +1399,14 @@
       <x:c r="D32" s="21"/>
       <x:c r="E32" s="21"/>
       <x:c r="F32" s="22"/>
-      <x:c r="G32" s="23"/>
-      <x:c r="H32" s="24"/>
+      <x:c r="G32" s="73"/>
+      <x:c r="H32" s="74"/>
+      <x:c r="I32" s="76"/>
+      <x:c r="J32" s="64"/>
+      <x:c r="K32" s="76"/>
+      <x:c r="L32" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="22" customHeight="1">
       <x:c r="A33" s="21" t="str">
@@ -1018,8 +1417,14 @@
       <x:c r="D33" s="21"/>
       <x:c r="E33" s="21"/>
       <x:c r="F33" s="22"/>
-      <x:c r="G33" s="23"/>
-      <x:c r="H33" s="24"/>
+      <x:c r="G33" s="73"/>
+      <x:c r="H33" s="74"/>
+      <x:c r="I33" s="76"/>
+      <x:c r="J33" s="64"/>
+      <x:c r="K33" s="76"/>
+      <x:c r="L33" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="22" customHeight="1">
       <x:c r="A34" s="21" t="str">
@@ -1030,8 +1435,14 @@
       <x:c r="D34" s="21"/>
       <x:c r="E34" s="21"/>
       <x:c r="F34" s="22"/>
-      <x:c r="G34" s="23"/>
-      <x:c r="H34" s="24"/>
+      <x:c r="G34" s="73"/>
+      <x:c r="H34" s="74"/>
+      <x:c r="I34" s="76"/>
+      <x:c r="J34" s="64"/>
+      <x:c r="K34" s="76"/>
+      <x:c r="L34" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="22" customHeight="1">
       <x:c r="A35" s="21" t="str">
@@ -1042,8 +1453,14 @@
       <x:c r="D35" s="21"/>
       <x:c r="E35" s="21"/>
       <x:c r="F35" s="22"/>
-      <x:c r="G35" s="23"/>
-      <x:c r="H35" s="24"/>
+      <x:c r="G35" s="73"/>
+      <x:c r="H35" s="74"/>
+      <x:c r="I35" s="76"/>
+      <x:c r="J35" s="64"/>
+      <x:c r="K35" s="76"/>
+      <x:c r="L35" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="22" customHeight="1">
       <x:c r="A36" s="21" t="str">
@@ -1054,8 +1471,14 @@
       <x:c r="D36" s="21"/>
       <x:c r="E36" s="21"/>
       <x:c r="F36" s="22"/>
-      <x:c r="G36" s="23"/>
-      <x:c r="H36" s="24"/>
+      <x:c r="G36" s="73"/>
+      <x:c r="H36" s="74"/>
+      <x:c r="I36" s="76"/>
+      <x:c r="J36" s="64"/>
+      <x:c r="K36" s="76"/>
+      <x:c r="L36" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="22" customHeight="1">
       <x:c r="A37" s="21" t="str">
@@ -1066,8 +1489,14 @@
       <x:c r="D37" s="21"/>
       <x:c r="E37" s="21"/>
       <x:c r="F37" s="22"/>
-      <x:c r="G37" s="23"/>
-      <x:c r="H37" s="24"/>
+      <x:c r="G37" s="73"/>
+      <x:c r="H37" s="74"/>
+      <x:c r="I37" s="76"/>
+      <x:c r="J37" s="64"/>
+      <x:c r="K37" s="76"/>
+      <x:c r="L37" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="22" customHeight="1">
       <x:c r="A38" s="21" t="str">
@@ -1078,8 +1507,14 @@
       <x:c r="D38" s="21"/>
       <x:c r="E38" s="21"/>
       <x:c r="F38" s="22"/>
-      <x:c r="G38" s="23"/>
-      <x:c r="H38" s="24"/>
+      <x:c r="G38" s="73"/>
+      <x:c r="H38" s="74"/>
+      <x:c r="I38" s="76"/>
+      <x:c r="J38" s="64"/>
+      <x:c r="K38" s="76"/>
+      <x:c r="L38" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="22" customHeight="1">
       <x:c r="A39" s="21" t="str">
@@ -1090,8 +1525,14 @@
       <x:c r="D39" s="21"/>
       <x:c r="E39" s="21"/>
       <x:c r="F39" s="22"/>
-      <x:c r="G39" s="23"/>
-      <x:c r="H39" s="24"/>
+      <x:c r="G39" s="73"/>
+      <x:c r="H39" s="74"/>
+      <x:c r="I39" s="76"/>
+      <x:c r="J39" s="64"/>
+      <x:c r="K39" s="76"/>
+      <x:c r="L39" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="22" customHeight="1">
       <x:c r="A40" s="21" t="str">
@@ -1102,8 +1543,14 @@
       <x:c r="D40" s="21"/>
       <x:c r="E40" s="21"/>
       <x:c r="F40" s="22"/>
-      <x:c r="G40" s="23"/>
-      <x:c r="H40" s="24"/>
+      <x:c r="G40" s="73"/>
+      <x:c r="H40" s="74"/>
+      <x:c r="I40" s="76"/>
+      <x:c r="J40" s="64"/>
+      <x:c r="K40" s="76"/>
+      <x:c r="L40" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="22" customHeight="1">
       <x:c r="A41" s="21" t="str">
@@ -1114,8 +1561,14 @@
       <x:c r="D41" s="21"/>
       <x:c r="E41" s="21"/>
       <x:c r="F41" s="22"/>
-      <x:c r="G41" s="23"/>
-      <x:c r="H41" s="24"/>
+      <x:c r="G41" s="73"/>
+      <x:c r="H41" s="74"/>
+      <x:c r="I41" s="76"/>
+      <x:c r="J41" s="64"/>
+      <x:c r="K41" s="76"/>
+      <x:c r="L41" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="22" customHeight="1">
       <x:c r="A42" s="21" t="str">
@@ -1126,8 +1579,14 @@
       <x:c r="D42" s="21"/>
       <x:c r="E42" s="21"/>
       <x:c r="F42" s="22"/>
-      <x:c r="G42" s="23"/>
-      <x:c r="H42" s="24"/>
+      <x:c r="G42" s="73"/>
+      <x:c r="H42" s="74"/>
+      <x:c r="I42" s="76"/>
+      <x:c r="J42" s="64"/>
+      <x:c r="K42" s="76"/>
+      <x:c r="L42" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="22" customHeight="1">
       <x:c r="A43" s="21" t="str">
@@ -1138,8 +1597,14 @@
       <x:c r="D43" s="21"/>
       <x:c r="E43" s="21"/>
       <x:c r="F43" s="22"/>
-      <x:c r="G43" s="23"/>
-      <x:c r="H43" s="24"/>
+      <x:c r="G43" s="73"/>
+      <x:c r="H43" s="74"/>
+      <x:c r="I43" s="76"/>
+      <x:c r="J43" s="64"/>
+      <x:c r="K43" s="76"/>
+      <x:c r="L43" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="22" customHeight="1">
       <x:c r="A44" s="21" t="str">
@@ -1150,8 +1615,14 @@
       <x:c r="D44" s="21"/>
       <x:c r="E44" s="21"/>
       <x:c r="F44" s="22"/>
-      <x:c r="G44" s="23"/>
-      <x:c r="H44" s="24"/>
+      <x:c r="G44" s="73"/>
+      <x:c r="H44" s="74"/>
+      <x:c r="I44" s="76"/>
+      <x:c r="J44" s="64"/>
+      <x:c r="K44" s="76"/>
+      <x:c r="L44" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="22" customHeight="1">
       <x:c r="A45" s="21" t="str">
@@ -1162,8 +1633,14 @@
       <x:c r="D45" s="21"/>
       <x:c r="E45" s="21"/>
       <x:c r="F45" s="22"/>
-      <x:c r="G45" s="23"/>
-      <x:c r="H45" s="24"/>
+      <x:c r="G45" s="73"/>
+      <x:c r="H45" s="74"/>
+      <x:c r="I45" s="76"/>
+      <x:c r="J45" s="64"/>
+      <x:c r="K45" s="76"/>
+      <x:c r="L45" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="22" customHeight="1">
       <x:c r="A46" s="21" t="str">
@@ -1174,8 +1651,14 @@
       <x:c r="D46" s="21"/>
       <x:c r="E46" s="21"/>
       <x:c r="F46" s="22"/>
-      <x:c r="G46" s="23"/>
-      <x:c r="H46" s="24"/>
+      <x:c r="G46" s="73"/>
+      <x:c r="H46" s="74"/>
+      <x:c r="I46" s="76"/>
+      <x:c r="J46" s="64"/>
+      <x:c r="K46" s="76"/>
+      <x:c r="L46" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="22" customHeight="1">
       <x:c r="A47" s="21" t="str">
@@ -1186,8 +1669,14 @@
       <x:c r="D47" s="21"/>
       <x:c r="E47" s="21"/>
       <x:c r="F47" s="22"/>
-      <x:c r="G47" s="23"/>
-      <x:c r="H47" s="24"/>
+      <x:c r="G47" s="73"/>
+      <x:c r="H47" s="74"/>
+      <x:c r="I47" s="76"/>
+      <x:c r="J47" s="64"/>
+      <x:c r="K47" s="76"/>
+      <x:c r="L47" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="22" customHeight="1">
       <x:c r="A48" s="21" t="str">
@@ -1198,8 +1687,14 @@
       <x:c r="D48" s="21"/>
       <x:c r="E48" s="21"/>
       <x:c r="F48" s="22"/>
-      <x:c r="G48" s="23"/>
-      <x:c r="H48" s="24"/>
+      <x:c r="G48" s="73"/>
+      <x:c r="H48" s="74"/>
+      <x:c r="I48" s="76"/>
+      <x:c r="J48" s="64"/>
+      <x:c r="K48" s="76"/>
+      <x:c r="L48" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="22" customHeight="1">
       <x:c r="A49" s="21" t="str">
@@ -1210,8 +1705,14 @@
       <x:c r="D49" s="21"/>
       <x:c r="E49" s="21"/>
       <x:c r="F49" s="22"/>
-      <x:c r="G49" s="23"/>
-      <x:c r="H49" s="24"/>
+      <x:c r="G49" s="73"/>
+      <x:c r="H49" s="74"/>
+      <x:c r="I49" s="76"/>
+      <x:c r="J49" s="64"/>
+      <x:c r="K49" s="76"/>
+      <x:c r="L49" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="22" customHeight="1">
       <x:c r="A50" s="21" t="str">
@@ -1222,8 +1723,14 @@
       <x:c r="D50" s="21"/>
       <x:c r="E50" s="21"/>
       <x:c r="F50" s="22"/>
-      <x:c r="G50" s="23"/>
-      <x:c r="H50" s="24"/>
+      <x:c r="G50" s="73"/>
+      <x:c r="H50" s="74"/>
+      <x:c r="I50" s="76"/>
+      <x:c r="J50" s="64"/>
+      <x:c r="K50" s="76"/>
+      <x:c r="L50" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="22" customHeight="1">
       <x:c r="A51" s="21" t="str">
@@ -1234,8 +1741,14 @@
       <x:c r="D51" s="21"/>
       <x:c r="E51" s="21"/>
       <x:c r="F51" s="22"/>
-      <x:c r="G51" s="23"/>
-      <x:c r="H51" s="24"/>
+      <x:c r="G51" s="73"/>
+      <x:c r="H51" s="74"/>
+      <x:c r="I51" s="76"/>
+      <x:c r="J51" s="64"/>
+      <x:c r="K51" s="76"/>
+      <x:c r="L51" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="22" customHeight="1">
       <x:c r="A52" s="21" t="str">
@@ -1246,8 +1759,14 @@
       <x:c r="D52" s="21"/>
       <x:c r="E52" s="21"/>
       <x:c r="F52" s="22"/>
-      <x:c r="G52" s="23"/>
-      <x:c r="H52" s="24"/>
+      <x:c r="G52" s="73"/>
+      <x:c r="H52" s="74"/>
+      <x:c r="I52" s="76"/>
+      <x:c r="J52" s="64"/>
+      <x:c r="K52" s="76"/>
+      <x:c r="L52" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="22" customHeight="1">
       <x:c r="A53" s="21" t="str">
@@ -1258,8 +1777,14 @@
       <x:c r="D53" s="21"/>
       <x:c r="E53" s="21"/>
       <x:c r="F53" s="22"/>
-      <x:c r="G53" s="23"/>
-      <x:c r="H53" s="24"/>
+      <x:c r="G53" s="73"/>
+      <x:c r="H53" s="74"/>
+      <x:c r="I53" s="76"/>
+      <x:c r="J53" s="64"/>
+      <x:c r="K53" s="76"/>
+      <x:c r="L53" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="22" customHeight="1">
       <x:c r="A54" s="21" t="str">
@@ -1270,8 +1795,14 @@
       <x:c r="D54" s="21"/>
       <x:c r="E54" s="21"/>
       <x:c r="F54" s="22"/>
-      <x:c r="G54" s="23"/>
-      <x:c r="H54" s="24"/>
+      <x:c r="G54" s="73"/>
+      <x:c r="H54" s="74"/>
+      <x:c r="I54" s="76"/>
+      <x:c r="J54" s="64"/>
+      <x:c r="K54" s="76"/>
+      <x:c r="L54" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="22" customHeight="1">
       <x:c r="A55" s="21" t="str">
@@ -1282,8 +1813,14 @@
       <x:c r="D55" s="21"/>
       <x:c r="E55" s="21"/>
       <x:c r="F55" s="22"/>
-      <x:c r="G55" s="23"/>
-      <x:c r="H55" s="24"/>
+      <x:c r="G55" s="73"/>
+      <x:c r="H55" s="74"/>
+      <x:c r="I55" s="76"/>
+      <x:c r="J55" s="64"/>
+      <x:c r="K55" s="76"/>
+      <x:c r="L55" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="22" customHeight="1">
       <x:c r="A56" s="21" t="str">
@@ -1294,8 +1831,14 @@
       <x:c r="D56" s="21"/>
       <x:c r="E56" s="21"/>
       <x:c r="F56" s="22"/>
-      <x:c r="G56" s="23"/>
-      <x:c r="H56" s="24"/>
+      <x:c r="G56" s="73"/>
+      <x:c r="H56" s="74"/>
+      <x:c r="I56" s="76"/>
+      <x:c r="J56" s="64"/>
+      <x:c r="K56" s="76"/>
+      <x:c r="L56" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="22" customHeight="1">
       <x:c r="A57" s="21" t="str">
@@ -1306,8 +1849,14 @@
       <x:c r="D57" s="21"/>
       <x:c r="E57" s="21"/>
       <x:c r="F57" s="22"/>
-      <x:c r="G57" s="23"/>
-      <x:c r="H57" s="24"/>
+      <x:c r="G57" s="73"/>
+      <x:c r="H57" s="74"/>
+      <x:c r="I57" s="76"/>
+      <x:c r="J57" s="64"/>
+      <x:c r="K57" s="76"/>
+      <x:c r="L57" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="22" customHeight="1">
       <x:c r="A58" s="21" t="str">
@@ -1318,8 +1867,14 @@
       <x:c r="D58" s="21"/>
       <x:c r="E58" s="21"/>
       <x:c r="F58" s="22"/>
-      <x:c r="G58" s="23"/>
-      <x:c r="H58" s="24"/>
+      <x:c r="G58" s="73"/>
+      <x:c r="H58" s="74"/>
+      <x:c r="I58" s="76"/>
+      <x:c r="J58" s="64"/>
+      <x:c r="K58" s="76"/>
+      <x:c r="L58" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="22" customHeight="1">
       <x:c r="A59" s="21" t="str">
@@ -1330,8 +1885,14 @@
       <x:c r="D59" s="21"/>
       <x:c r="E59" s="21"/>
       <x:c r="F59" s="22"/>
-      <x:c r="G59" s="23"/>
-      <x:c r="H59" s="24"/>
+      <x:c r="G59" s="73"/>
+      <x:c r="H59" s="74"/>
+      <x:c r="I59" s="76"/>
+      <x:c r="J59" s="64"/>
+      <x:c r="K59" s="76"/>
+      <x:c r="L59" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="22" customHeight="1">
       <x:c r="A60" s="21" t="str">
@@ -1342,8 +1903,14 @@
       <x:c r="D60" s="21"/>
       <x:c r="E60" s="21"/>
       <x:c r="F60" s="22"/>
-      <x:c r="G60" s="23"/>
-      <x:c r="H60" s="24"/>
+      <x:c r="G60" s="73"/>
+      <x:c r="H60" s="74"/>
+      <x:c r="I60" s="76"/>
+      <x:c r="J60" s="64"/>
+      <x:c r="K60" s="76"/>
+      <x:c r="L60" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="22" customHeight="1">
       <x:c r="A61" s="21" t="str">
@@ -1354,8 +1921,14 @@
       <x:c r="D61" s="21"/>
       <x:c r="E61" s="21"/>
       <x:c r="F61" s="22"/>
-      <x:c r="G61" s="23"/>
-      <x:c r="H61" s="24"/>
+      <x:c r="G61" s="73"/>
+      <x:c r="H61" s="74"/>
+      <x:c r="I61" s="76"/>
+      <x:c r="J61" s="64"/>
+      <x:c r="K61" s="76"/>
+      <x:c r="L61" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="22" customHeight="1">
       <x:c r="A62" s="21" t="str">
@@ -1366,8 +1939,14 @@
       <x:c r="D62" s="21"/>
       <x:c r="E62" s="21"/>
       <x:c r="F62" s="22"/>
-      <x:c r="G62" s="23"/>
-      <x:c r="H62" s="24"/>
+      <x:c r="G62" s="73"/>
+      <x:c r="H62" s="74"/>
+      <x:c r="I62" s="76"/>
+      <x:c r="J62" s="64"/>
+      <x:c r="K62" s="76"/>
+      <x:c r="L62" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="22" customHeight="1">
       <x:c r="A63" s="21" t="str">
@@ -1378,8 +1957,14 @@
       <x:c r="D63" s="21"/>
       <x:c r="E63" s="21"/>
       <x:c r="F63" s="22"/>
-      <x:c r="G63" s="23"/>
-      <x:c r="H63" s="24"/>
+      <x:c r="G63" s="73"/>
+      <x:c r="H63" s="74"/>
+      <x:c r="I63" s="76"/>
+      <x:c r="J63" s="64"/>
+      <x:c r="K63" s="76"/>
+      <x:c r="L63" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="22" customHeight="1">
       <x:c r="A64" s="21" t="str">
@@ -1390,8 +1975,14 @@
       <x:c r="D64" s="21"/>
       <x:c r="E64" s="21"/>
       <x:c r="F64" s="22"/>
-      <x:c r="G64" s="23"/>
-      <x:c r="H64" s="24"/>
+      <x:c r="G64" s="73"/>
+      <x:c r="H64" s="74"/>
+      <x:c r="I64" s="76"/>
+      <x:c r="J64" s="64"/>
+      <x:c r="K64" s="76"/>
+      <x:c r="L64" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="22" customHeight="1">
       <x:c r="A65" s="21" t="str">
@@ -1402,8 +1993,14 @@
       <x:c r="D65" s="21"/>
       <x:c r="E65" s="21"/>
       <x:c r="F65" s="22"/>
-      <x:c r="G65" s="23"/>
-      <x:c r="H65" s="24"/>
+      <x:c r="G65" s="73"/>
+      <x:c r="H65" s="74"/>
+      <x:c r="I65" s="76"/>
+      <x:c r="J65" s="64"/>
+      <x:c r="K65" s="76"/>
+      <x:c r="L65" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="22" customHeight="1">
       <x:c r="A66" s="21" t="str">
@@ -1414,8 +2011,14 @@
       <x:c r="D66" s="21"/>
       <x:c r="E66" s="21"/>
       <x:c r="F66" s="22"/>
-      <x:c r="G66" s="23"/>
-      <x:c r="H66" s="24"/>
+      <x:c r="G66" s="73"/>
+      <x:c r="H66" s="74"/>
+      <x:c r="I66" s="76"/>
+      <x:c r="J66" s="64"/>
+      <x:c r="K66" s="76"/>
+      <x:c r="L66" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="22" customHeight="1">
       <x:c r="A67" s="21" t="str">
@@ -1426,8 +2029,14 @@
       <x:c r="D67" s="21"/>
       <x:c r="E67" s="21"/>
       <x:c r="F67" s="22"/>
-      <x:c r="G67" s="23"/>
-      <x:c r="H67" s="24"/>
+      <x:c r="G67" s="73"/>
+      <x:c r="H67" s="74"/>
+      <x:c r="I67" s="76"/>
+      <x:c r="J67" s="64"/>
+      <x:c r="K67" s="76"/>
+      <x:c r="L67" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="22" customHeight="1">
       <x:c r="A68" s="21" t="str">
@@ -1438,8 +2047,14 @@
       <x:c r="D68" s="21"/>
       <x:c r="E68" s="21"/>
       <x:c r="F68" s="22"/>
-      <x:c r="G68" s="23"/>
-      <x:c r="H68" s="24"/>
+      <x:c r="G68" s="73"/>
+      <x:c r="H68" s="74"/>
+      <x:c r="I68" s="76"/>
+      <x:c r="J68" s="64"/>
+      <x:c r="K68" s="76"/>
+      <x:c r="L68" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="22" customHeight="1">
       <x:c r="A69" s="21" t="str">
@@ -1450,8 +2065,14 @@
       <x:c r="D69" s="21"/>
       <x:c r="E69" s="21"/>
       <x:c r="F69" s="22"/>
-      <x:c r="G69" s="23"/>
-      <x:c r="H69" s="24"/>
+      <x:c r="G69" s="73"/>
+      <x:c r="H69" s="74"/>
+      <x:c r="I69" s="76"/>
+      <x:c r="J69" s="64"/>
+      <x:c r="K69" s="76"/>
+      <x:c r="L69" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="22" customHeight="1">
       <x:c r="A70" s="21" t="str">
@@ -1462,8 +2083,14 @@
       <x:c r="D70" s="21"/>
       <x:c r="E70" s="21"/>
       <x:c r="F70" s="22"/>
-      <x:c r="G70" s="23"/>
-      <x:c r="H70" s="24"/>
+      <x:c r="G70" s="73"/>
+      <x:c r="H70" s="74"/>
+      <x:c r="I70" s="76"/>
+      <x:c r="J70" s="64"/>
+      <x:c r="K70" s="76"/>
+      <x:c r="L70" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="22" customHeight="1">
       <x:c r="A71" s="21" t="str">
@@ -1474,8 +2101,14 @@
       <x:c r="D71" s="21"/>
       <x:c r="E71" s="21"/>
       <x:c r="F71" s="22"/>
-      <x:c r="G71" s="23"/>
-      <x:c r="H71" s="24"/>
+      <x:c r="G71" s="73"/>
+      <x:c r="H71" s="74"/>
+      <x:c r="I71" s="76"/>
+      <x:c r="J71" s="64"/>
+      <x:c r="K71" s="76"/>
+      <x:c r="L71" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" ht="22" customHeight="1">
       <x:c r="A72" s="21" t="str">
@@ -1486,8 +2119,14 @@
       <x:c r="D72" s="21"/>
       <x:c r="E72" s="21"/>
       <x:c r="F72" s="22"/>
-      <x:c r="G72" s="23"/>
-      <x:c r="H72" s="24"/>
+      <x:c r="G72" s="73"/>
+      <x:c r="H72" s="74"/>
+      <x:c r="I72" s="76"/>
+      <x:c r="J72" s="64"/>
+      <x:c r="K72" s="76"/>
+      <x:c r="L72" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" ht="22" customHeight="1">
       <x:c r="A73" s="21" t="str">
@@ -1498,8 +2137,14 @@
       <x:c r="D73" s="21"/>
       <x:c r="E73" s="21"/>
       <x:c r="F73" s="22"/>
-      <x:c r="G73" s="23"/>
-      <x:c r="H73" s="24"/>
+      <x:c r="G73" s="73"/>
+      <x:c r="H73" s="74"/>
+      <x:c r="I73" s="76"/>
+      <x:c r="J73" s="64"/>
+      <x:c r="K73" s="76"/>
+      <x:c r="L73" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="22" customHeight="1">
       <x:c r="A74" s="21" t="str">
@@ -1510,8 +2155,14 @@
       <x:c r="D74" s="21"/>
       <x:c r="E74" s="21"/>
       <x:c r="F74" s="22"/>
-      <x:c r="G74" s="23"/>
-      <x:c r="H74" s="24"/>
+      <x:c r="G74" s="73"/>
+      <x:c r="H74" s="74"/>
+      <x:c r="I74" s="76"/>
+      <x:c r="J74" s="64"/>
+      <x:c r="K74" s="76"/>
+      <x:c r="L74" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" ht="22" customHeight="1">
       <x:c r="A75" s="21" t="str">
@@ -1522,8 +2173,14 @@
       <x:c r="D75" s="21"/>
       <x:c r="E75" s="21"/>
       <x:c r="F75" s="22"/>
-      <x:c r="G75" s="23"/>
-      <x:c r="H75" s="24"/>
+      <x:c r="G75" s="73"/>
+      <x:c r="H75" s="74"/>
+      <x:c r="I75" s="76"/>
+      <x:c r="J75" s="64"/>
+      <x:c r="K75" s="76"/>
+      <x:c r="L75" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="76" ht="22" customHeight="1">
       <x:c r="A76" s="21" t="str">
@@ -1534,8 +2191,14 @@
       <x:c r="D76" s="21"/>
       <x:c r="E76" s="21"/>
       <x:c r="F76" s="22"/>
-      <x:c r="G76" s="23"/>
-      <x:c r="H76" s="24"/>
+      <x:c r="G76" s="73"/>
+      <x:c r="H76" s="74"/>
+      <x:c r="I76" s="76"/>
+      <x:c r="J76" s="64"/>
+      <x:c r="K76" s="76"/>
+      <x:c r="L76" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" ht="22" customHeight="1">
       <x:c r="A77" s="21" t="str">
@@ -1546,8 +2209,14 @@
       <x:c r="D77" s="21"/>
       <x:c r="E77" s="21"/>
       <x:c r="F77" s="22"/>
-      <x:c r="G77" s="23"/>
-      <x:c r="H77" s="24"/>
+      <x:c r="G77" s="73"/>
+      <x:c r="H77" s="74"/>
+      <x:c r="I77" s="76"/>
+      <x:c r="J77" s="64"/>
+      <x:c r="K77" s="76"/>
+      <x:c r="L77" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="78" ht="22" customHeight="1">
       <x:c r="A78" s="21" t="str">
@@ -1558,8 +2227,14 @@
       <x:c r="D78" s="21"/>
       <x:c r="E78" s="21"/>
       <x:c r="F78" s="22"/>
-      <x:c r="G78" s="23"/>
-      <x:c r="H78" s="24"/>
+      <x:c r="G78" s="73"/>
+      <x:c r="H78" s="74"/>
+      <x:c r="I78" s="76"/>
+      <x:c r="J78" s="64"/>
+      <x:c r="K78" s="76"/>
+      <x:c r="L78" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="79" ht="22" customHeight="1">
       <x:c r="A79" s="21" t="str">
@@ -1570,8 +2245,14 @@
       <x:c r="D79" s="21"/>
       <x:c r="E79" s="21"/>
       <x:c r="F79" s="22"/>
-      <x:c r="G79" s="23"/>
-      <x:c r="H79" s="24"/>
+      <x:c r="G79" s="73"/>
+      <x:c r="H79" s="74"/>
+      <x:c r="I79" s="76"/>
+      <x:c r="J79" s="64"/>
+      <x:c r="K79" s="76"/>
+      <x:c r="L79" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="80" ht="22" customHeight="1">
       <x:c r="A80" s="21" t="str">
@@ -1582,8 +2263,14 @@
       <x:c r="D80" s="21"/>
       <x:c r="E80" s="21"/>
       <x:c r="F80" s="22"/>
-      <x:c r="G80" s="23"/>
-      <x:c r="H80" s="24"/>
+      <x:c r="G80" s="73"/>
+      <x:c r="H80" s="74"/>
+      <x:c r="I80" s="76"/>
+      <x:c r="J80" s="64"/>
+      <x:c r="K80" s="76"/>
+      <x:c r="L80" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="81" ht="22" customHeight="1">
       <x:c r="A81" s="21" t="str">
@@ -1594,8 +2281,14 @@
       <x:c r="D81" s="21"/>
       <x:c r="E81" s="21"/>
       <x:c r="F81" s="22"/>
-      <x:c r="G81" s="23"/>
-      <x:c r="H81" s="24"/>
+      <x:c r="G81" s="73"/>
+      <x:c r="H81" s="74"/>
+      <x:c r="I81" s="76"/>
+      <x:c r="J81" s="64"/>
+      <x:c r="K81" s="76"/>
+      <x:c r="L81" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="82" ht="22" customHeight="1">
       <x:c r="A82" s="21" t="str">
@@ -1606,8 +2299,14 @@
       <x:c r="D82" s="21"/>
       <x:c r="E82" s="21"/>
       <x:c r="F82" s="22"/>
-      <x:c r="G82" s="23"/>
-      <x:c r="H82" s="24"/>
+      <x:c r="G82" s="73"/>
+      <x:c r="H82" s="74"/>
+      <x:c r="I82" s="76"/>
+      <x:c r="J82" s="64"/>
+      <x:c r="K82" s="76"/>
+      <x:c r="L82" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="83" ht="22" customHeight="1">
       <x:c r="A83" s="21" t="str">
@@ -1618,8 +2317,14 @@
       <x:c r="D83" s="21"/>
       <x:c r="E83" s="21"/>
       <x:c r="F83" s="22"/>
-      <x:c r="G83" s="23"/>
-      <x:c r="H83" s="24"/>
+      <x:c r="G83" s="73"/>
+      <x:c r="H83" s="74"/>
+      <x:c r="I83" s="76"/>
+      <x:c r="J83" s="64"/>
+      <x:c r="K83" s="76"/>
+      <x:c r="L83" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="84" ht="22" customHeight="1">
       <x:c r="A84" s="21" t="str">
@@ -1630,8 +2335,14 @@
       <x:c r="D84" s="21"/>
       <x:c r="E84" s="21"/>
       <x:c r="F84" s="22"/>
-      <x:c r="G84" s="23"/>
-      <x:c r="H84" s="24"/>
+      <x:c r="G84" s="73"/>
+      <x:c r="H84" s="74"/>
+      <x:c r="I84" s="76"/>
+      <x:c r="J84" s="64"/>
+      <x:c r="K84" s="76"/>
+      <x:c r="L84" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="85" ht="22" customHeight="1">
       <x:c r="A85" s="21" t="str">
@@ -1642,8 +2353,14 @@
       <x:c r="D85" s="21"/>
       <x:c r="E85" s="21"/>
       <x:c r="F85" s="22"/>
-      <x:c r="G85" s="23"/>
-      <x:c r="H85" s="24"/>
+      <x:c r="G85" s="73"/>
+      <x:c r="H85" s="74"/>
+      <x:c r="I85" s="76"/>
+      <x:c r="J85" s="64"/>
+      <x:c r="K85" s="76"/>
+      <x:c r="L85" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="86" ht="22" customHeight="1">
       <x:c r="A86" s="21" t="str">
@@ -1654,8 +2371,14 @@
       <x:c r="D86" s="21"/>
       <x:c r="E86" s="21"/>
       <x:c r="F86" s="22"/>
-      <x:c r="G86" s="23"/>
-      <x:c r="H86" s="24"/>
+      <x:c r="G86" s="73"/>
+      <x:c r="H86" s="74"/>
+      <x:c r="I86" s="76"/>
+      <x:c r="J86" s="64"/>
+      <x:c r="K86" s="76"/>
+      <x:c r="L86" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="87" ht="22" customHeight="1">
       <x:c r="A87" s="21" t="str">
@@ -1666,8 +2389,14 @@
       <x:c r="D87" s="21"/>
       <x:c r="E87" s="21"/>
       <x:c r="F87" s="22"/>
-      <x:c r="G87" s="23"/>
-      <x:c r="H87" s="24"/>
+      <x:c r="G87" s="73"/>
+      <x:c r="H87" s="74"/>
+      <x:c r="I87" s="76"/>
+      <x:c r="J87" s="64"/>
+      <x:c r="K87" s="76"/>
+      <x:c r="L87" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="88" ht="22" customHeight="1">
       <x:c r="A88" s="21" t="str">
@@ -1678,8 +2407,14 @@
       <x:c r="D88" s="21"/>
       <x:c r="E88" s="21"/>
       <x:c r="F88" s="22"/>
-      <x:c r="G88" s="23"/>
-      <x:c r="H88" s="24"/>
+      <x:c r="G88" s="73"/>
+      <x:c r="H88" s="74"/>
+      <x:c r="I88" s="76"/>
+      <x:c r="J88" s="64"/>
+      <x:c r="K88" s="76"/>
+      <x:c r="L88" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="89" ht="22" customHeight="1">
       <x:c r="A89" s="21" t="str">
@@ -1690,8 +2425,14 @@
       <x:c r="D89" s="21"/>
       <x:c r="E89" s="21"/>
       <x:c r="F89" s="22"/>
-      <x:c r="G89" s="23"/>
-      <x:c r="H89" s="24"/>
+      <x:c r="G89" s="73"/>
+      <x:c r="H89" s="74"/>
+      <x:c r="I89" s="76"/>
+      <x:c r="J89" s="64"/>
+      <x:c r="K89" s="76"/>
+      <x:c r="L89" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="90" ht="22" customHeight="1">
       <x:c r="A90" s="21" t="str">
@@ -1702,8 +2443,14 @@
       <x:c r="D90" s="21"/>
       <x:c r="E90" s="21"/>
       <x:c r="F90" s="22"/>
-      <x:c r="G90" s="23"/>
-      <x:c r="H90" s="24"/>
+      <x:c r="G90" s="73"/>
+      <x:c r="H90" s="74"/>
+      <x:c r="I90" s="76"/>
+      <x:c r="J90" s="64"/>
+      <x:c r="K90" s="76"/>
+      <x:c r="L90" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="91" ht="22" customHeight="1">
       <x:c r="A91" s="21" t="str">
@@ -1714,8 +2461,14 @@
       <x:c r="D91" s="21"/>
       <x:c r="E91" s="21"/>
       <x:c r="F91" s="22"/>
-      <x:c r="G91" s="23"/>
-      <x:c r="H91" s="24"/>
+      <x:c r="G91" s="73"/>
+      <x:c r="H91" s="74"/>
+      <x:c r="I91" s="76"/>
+      <x:c r="J91" s="64"/>
+      <x:c r="K91" s="76"/>
+      <x:c r="L91" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="92" ht="22" customHeight="1">
       <x:c r="A92" s="21" t="str">
@@ -1726,8 +2479,14 @@
       <x:c r="D92" s="21"/>
       <x:c r="E92" s="21"/>
       <x:c r="F92" s="22"/>
-      <x:c r="G92" s="23"/>
-      <x:c r="H92" s="24"/>
+      <x:c r="G92" s="73"/>
+      <x:c r="H92" s="74"/>
+      <x:c r="I92" s="76"/>
+      <x:c r="J92" s="64"/>
+      <x:c r="K92" s="76"/>
+      <x:c r="L92" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="93" ht="22" customHeight="1">
       <x:c r="A93" s="21" t="str">
@@ -1738,8 +2497,14 @@
       <x:c r="D93" s="21"/>
       <x:c r="E93" s="21"/>
       <x:c r="F93" s="22"/>
-      <x:c r="G93" s="23"/>
-      <x:c r="H93" s="24"/>
+      <x:c r="G93" s="73"/>
+      <x:c r="H93" s="74"/>
+      <x:c r="I93" s="76"/>
+      <x:c r="J93" s="64"/>
+      <x:c r="K93" s="76"/>
+      <x:c r="L93" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="94" ht="22" customHeight="1">
       <x:c r="A94" s="21" t="str">
@@ -1750,8 +2515,14 @@
       <x:c r="D94" s="21"/>
       <x:c r="E94" s="21"/>
       <x:c r="F94" s="22"/>
-      <x:c r="G94" s="23"/>
-      <x:c r="H94" s="24"/>
+      <x:c r="G94" s="73"/>
+      <x:c r="H94" s="74"/>
+      <x:c r="I94" s="76"/>
+      <x:c r="J94" s="64"/>
+      <x:c r="K94" s="76"/>
+      <x:c r="L94" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="95" ht="22" customHeight="1">
       <x:c r="A95" s="21" t="str">
@@ -1762,8 +2533,14 @@
       <x:c r="D95" s="21"/>
       <x:c r="E95" s="21"/>
       <x:c r="F95" s="22"/>
-      <x:c r="G95" s="23"/>
-      <x:c r="H95" s="24"/>
+      <x:c r="G95" s="73"/>
+      <x:c r="H95" s="74"/>
+      <x:c r="I95" s="76"/>
+      <x:c r="J95" s="64"/>
+      <x:c r="K95" s="76"/>
+      <x:c r="L95" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="96" ht="22" customHeight="1">
       <x:c r="A96" s="21" t="str">
@@ -1774,8 +2551,14 @@
       <x:c r="D96" s="21"/>
       <x:c r="E96" s="21"/>
       <x:c r="F96" s="22"/>
-      <x:c r="G96" s="23"/>
-      <x:c r="H96" s="24"/>
+      <x:c r="G96" s="73"/>
+      <x:c r="H96" s="74"/>
+      <x:c r="I96" s="76"/>
+      <x:c r="J96" s="64"/>
+      <x:c r="K96" s="76"/>
+      <x:c r="L96" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="97" ht="22" customHeight="1">
       <x:c r="A97" s="21" t="str">
@@ -1786,8 +2569,14 @@
       <x:c r="D97" s="21"/>
       <x:c r="E97" s="21"/>
       <x:c r="F97" s="22"/>
-      <x:c r="G97" s="23"/>
-      <x:c r="H97" s="24"/>
+      <x:c r="G97" s="73"/>
+      <x:c r="H97" s="74"/>
+      <x:c r="I97" s="76"/>
+      <x:c r="J97" s="64"/>
+      <x:c r="K97" s="76"/>
+      <x:c r="L97" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="98" ht="22" customHeight="1">
       <x:c r="A98" s="21" t="str">
@@ -1798,8 +2587,14 @@
       <x:c r="D98" s="21"/>
       <x:c r="E98" s="21"/>
       <x:c r="F98" s="22"/>
-      <x:c r="G98" s="23"/>
-      <x:c r="H98" s="24"/>
+      <x:c r="G98" s="73"/>
+      <x:c r="H98" s="74"/>
+      <x:c r="I98" s="76"/>
+      <x:c r="J98" s="64"/>
+      <x:c r="K98" s="76"/>
+      <x:c r="L98" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="99" ht="22" customHeight="1">
       <x:c r="A99" s="21" t="str">
@@ -1810,8 +2605,14 @@
       <x:c r="D99" s="21"/>
       <x:c r="E99" s="21"/>
       <x:c r="F99" s="22"/>
-      <x:c r="G99" s="23"/>
-      <x:c r="H99" s="24"/>
+      <x:c r="G99" s="73"/>
+      <x:c r="H99" s="74"/>
+      <x:c r="I99" s="76"/>
+      <x:c r="J99" s="64"/>
+      <x:c r="K99" s="76"/>
+      <x:c r="L99" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="100" ht="22" customHeight="1">
       <x:c r="A100" s="21" t="str">
@@ -1822,8 +2623,14 @@
       <x:c r="D100" s="21"/>
       <x:c r="E100" s="21"/>
       <x:c r="F100" s="22"/>
-      <x:c r="G100" s="23"/>
-      <x:c r="H100" s="24"/>
+      <x:c r="G100" s="73"/>
+      <x:c r="H100" s="74"/>
+      <x:c r="I100" s="76"/>
+      <x:c r="J100" s="64"/>
+      <x:c r="K100" s="76"/>
+      <x:c r="L100" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="101" ht="22" customHeight="1">
       <x:c r="A101" s="21" t="str">
@@ -1834,8 +2641,14 @@
       <x:c r="D101" s="21"/>
       <x:c r="E101" s="21"/>
       <x:c r="F101" s="22"/>
-      <x:c r="G101" s="23"/>
-      <x:c r="H101" s="24"/>
+      <x:c r="G101" s="73"/>
+      <x:c r="H101" s="74"/>
+      <x:c r="I101" s="76"/>
+      <x:c r="J101" s="64"/>
+      <x:c r="K101" s="76"/>
+      <x:c r="L101" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="102" ht="22" customHeight="1">
       <x:c r="A102" s="21" t="str">
@@ -1846,8 +2659,14 @@
       <x:c r="D102" s="21"/>
       <x:c r="E102" s="21"/>
       <x:c r="F102" s="22"/>
-      <x:c r="G102" s="23"/>
-      <x:c r="H102" s="24"/>
+      <x:c r="G102" s="73"/>
+      <x:c r="H102" s="74"/>
+      <x:c r="I102" s="76"/>
+      <x:c r="J102" s="64"/>
+      <x:c r="K102" s="76"/>
+      <x:c r="L102" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="103" ht="22" customHeight="1">
       <x:c r="A103" s="21" t="str">
@@ -1858,8 +2677,14 @@
       <x:c r="D103" s="21"/>
       <x:c r="E103" s="21"/>
       <x:c r="F103" s="22"/>
-      <x:c r="G103" s="23"/>
-      <x:c r="H103" s="24"/>
+      <x:c r="G103" s="73"/>
+      <x:c r="H103" s="74"/>
+      <x:c r="I103" s="76"/>
+      <x:c r="J103" s="64"/>
+      <x:c r="K103" s="76"/>
+      <x:c r="L103" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="104" ht="22" customHeight="1">
       <x:c r="A104" s="21" t="str">
@@ -1870,8 +2695,14 @@
       <x:c r="D104" s="21"/>
       <x:c r="E104" s="21"/>
       <x:c r="F104" s="22"/>
-      <x:c r="G104" s="23"/>
-      <x:c r="H104" s="24"/>
+      <x:c r="G104" s="73"/>
+      <x:c r="H104" s="74"/>
+      <x:c r="I104" s="76"/>
+      <x:c r="J104" s="64"/>
+      <x:c r="K104" s="76"/>
+      <x:c r="L104" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="105" ht="22" customHeight="1">
       <x:c r="A105" s="21" t="str">
@@ -1882,8 +2713,14 @@
       <x:c r="D105" s="21"/>
       <x:c r="E105" s="21"/>
       <x:c r="F105" s="22"/>
-      <x:c r="G105" s="23"/>
-      <x:c r="H105" s="24"/>
+      <x:c r="G105" s="73"/>
+      <x:c r="H105" s="74"/>
+      <x:c r="I105" s="76"/>
+      <x:c r="J105" s="64"/>
+      <x:c r="K105" s="76"/>
+      <x:c r="L105" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="106" ht="22" customHeight="1">
       <x:c r="A106" s="21" t="str">
@@ -1894,8 +2731,14 @@
       <x:c r="D106" s="21"/>
       <x:c r="E106" s="21"/>
       <x:c r="F106" s="22"/>
-      <x:c r="G106" s="23"/>
-      <x:c r="H106" s="24"/>
+      <x:c r="G106" s="73"/>
+      <x:c r="H106" s="74"/>
+      <x:c r="I106" s="76"/>
+      <x:c r="J106" s="64"/>
+      <x:c r="K106" s="76"/>
+      <x:c r="L106" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="107" ht="22" customHeight="1">
       <x:c r="A107" s="21" t="str">
@@ -1906,8 +2749,14 @@
       <x:c r="D107" s="21"/>
       <x:c r="E107" s="21"/>
       <x:c r="F107" s="22"/>
-      <x:c r="G107" s="23"/>
-      <x:c r="H107" s="24"/>
+      <x:c r="G107" s="73"/>
+      <x:c r="H107" s="74"/>
+      <x:c r="I107" s="76"/>
+      <x:c r="J107" s="64"/>
+      <x:c r="K107" s="76"/>
+      <x:c r="L107" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="108" ht="22" customHeight="1">
       <x:c r="A108" s="21" t="str">
@@ -1918,8 +2767,14 @@
       <x:c r="D108" s="21"/>
       <x:c r="E108" s="21"/>
       <x:c r="F108" s="22"/>
-      <x:c r="G108" s="23"/>
-      <x:c r="H108" s="24"/>
+      <x:c r="G108" s="73"/>
+      <x:c r="H108" s="74"/>
+      <x:c r="I108" s="76"/>
+      <x:c r="J108" s="64"/>
+      <x:c r="K108" s="76"/>
+      <x:c r="L108" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="109" ht="22" customHeight="1">
       <x:c r="A109" s="21" t="str">
@@ -1930,8 +2785,14 @@
       <x:c r="D109" s="21"/>
       <x:c r="E109" s="21"/>
       <x:c r="F109" s="22"/>
-      <x:c r="G109" s="23"/>
-      <x:c r="H109" s="24"/>
+      <x:c r="G109" s="73"/>
+      <x:c r="H109" s="74"/>
+      <x:c r="I109" s="76"/>
+      <x:c r="J109" s="64"/>
+      <x:c r="K109" s="76"/>
+      <x:c r="L109" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="110" ht="22" customHeight="1">
       <x:c r="A110" s="21" t="str">
@@ -1942,8 +2803,14 @@
       <x:c r="D110" s="21"/>
       <x:c r="E110" s="21"/>
       <x:c r="F110" s="22"/>
-      <x:c r="G110" s="23"/>
-      <x:c r="H110" s="24"/>
+      <x:c r="G110" s="73"/>
+      <x:c r="H110" s="74"/>
+      <x:c r="I110" s="76"/>
+      <x:c r="J110" s="64"/>
+      <x:c r="K110" s="76"/>
+      <x:c r="L110" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="111" ht="22" customHeight="1">
       <x:c r="A111" s="21" t="str">
@@ -1954,8 +2821,14 @@
       <x:c r="D111" s="21"/>
       <x:c r="E111" s="21"/>
       <x:c r="F111" s="22"/>
-      <x:c r="G111" s="23"/>
-      <x:c r="H111" s="24"/>
+      <x:c r="G111" s="73"/>
+      <x:c r="H111" s="74"/>
+      <x:c r="I111" s="76"/>
+      <x:c r="J111" s="64"/>
+      <x:c r="K111" s="76"/>
+      <x:c r="L111" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="112" ht="22" customHeight="1">
       <x:c r="A112" s="21" t="str">
@@ -1966,8 +2839,14 @@
       <x:c r="D112" s="21"/>
       <x:c r="E112" s="21"/>
       <x:c r="F112" s="22"/>
-      <x:c r="G112" s="23"/>
-      <x:c r="H112" s="24"/>
+      <x:c r="G112" s="73"/>
+      <x:c r="H112" s="74"/>
+      <x:c r="I112" s="76"/>
+      <x:c r="J112" s="64"/>
+      <x:c r="K112" s="76"/>
+      <x:c r="L112" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="113" ht="22" customHeight="1">
       <x:c r="A113" s="21" t="str">
@@ -1978,8 +2857,14 @@
       <x:c r="D113" s="21"/>
       <x:c r="E113" s="21"/>
       <x:c r="F113" s="22"/>
-      <x:c r="G113" s="23"/>
-      <x:c r="H113" s="24"/>
+      <x:c r="G113" s="73"/>
+      <x:c r="H113" s="74"/>
+      <x:c r="I113" s="76"/>
+      <x:c r="J113" s="64"/>
+      <x:c r="K113" s="76"/>
+      <x:c r="L113" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="114" ht="22" customHeight="1">
       <x:c r="A114" s="21" t="str">
@@ -1990,8 +2875,14 @@
       <x:c r="D114" s="21"/>
       <x:c r="E114" s="21"/>
       <x:c r="F114" s="22"/>
-      <x:c r="G114" s="23"/>
-      <x:c r="H114" s="24"/>
+      <x:c r="G114" s="73"/>
+      <x:c r="H114" s="74"/>
+      <x:c r="I114" s="76"/>
+      <x:c r="J114" s="64"/>
+      <x:c r="K114" s="76"/>
+      <x:c r="L114" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="115" ht="22" customHeight="1">
       <x:c r="A115" s="21" t="str">
@@ -2002,8 +2893,14 @@
       <x:c r="D115" s="21"/>
       <x:c r="E115" s="21"/>
       <x:c r="F115" s="22"/>
-      <x:c r="G115" s="23"/>
-      <x:c r="H115" s="24"/>
+      <x:c r="G115" s="73"/>
+      <x:c r="H115" s="74"/>
+      <x:c r="I115" s="76"/>
+      <x:c r="J115" s="64"/>
+      <x:c r="K115" s="76"/>
+      <x:c r="L115" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="116" ht="22" customHeight="1">
       <x:c r="A116" s="21" t="str">
@@ -2014,8 +2911,14 @@
       <x:c r="D116" s="21"/>
       <x:c r="E116" s="21"/>
       <x:c r="F116" s="22"/>
-      <x:c r="G116" s="23"/>
-      <x:c r="H116" s="24"/>
+      <x:c r="G116" s="73"/>
+      <x:c r="H116" s="74"/>
+      <x:c r="I116" s="76"/>
+      <x:c r="J116" s="64"/>
+      <x:c r="K116" s="76"/>
+      <x:c r="L116" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="117" ht="22" customHeight="1">
       <x:c r="A117" s="21" t="str">
@@ -2026,8 +2929,14 @@
       <x:c r="D117" s="21"/>
       <x:c r="E117" s="21"/>
       <x:c r="F117" s="22"/>
-      <x:c r="G117" s="23"/>
-      <x:c r="H117" s="24"/>
+      <x:c r="G117" s="73"/>
+      <x:c r="H117" s="74"/>
+      <x:c r="I117" s="76"/>
+      <x:c r="J117" s="64"/>
+      <x:c r="K117" s="76"/>
+      <x:c r="L117" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="118" ht="22" customHeight="1">
       <x:c r="A118" s="21" t="str">
@@ -2038,8 +2947,14 @@
       <x:c r="D118" s="21"/>
       <x:c r="E118" s="21"/>
       <x:c r="F118" s="22"/>
-      <x:c r="G118" s="23"/>
-      <x:c r="H118" s="24"/>
+      <x:c r="G118" s="73"/>
+      <x:c r="H118" s="74"/>
+      <x:c r="I118" s="76"/>
+      <x:c r="J118" s="64"/>
+      <x:c r="K118" s="76"/>
+      <x:c r="L118" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="119" ht="22" customHeight="1">
       <x:c r="A119" s="21" t="str">
@@ -2050,8 +2965,14 @@
       <x:c r="D119" s="21"/>
       <x:c r="E119" s="21"/>
       <x:c r="F119" s="22"/>
-      <x:c r="G119" s="23"/>
-      <x:c r="H119" s="24"/>
+      <x:c r="G119" s="73"/>
+      <x:c r="H119" s="74"/>
+      <x:c r="I119" s="76"/>
+      <x:c r="J119" s="64"/>
+      <x:c r="K119" s="76"/>
+      <x:c r="L119" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="120" ht="22" customHeight="1">
       <x:c r="A120" s="21" t="str">
@@ -2062,8 +2983,14 @@
       <x:c r="D120" s="21"/>
       <x:c r="E120" s="21"/>
       <x:c r="F120" s="22"/>
-      <x:c r="G120" s="23"/>
-      <x:c r="H120" s="24"/>
+      <x:c r="G120" s="73"/>
+      <x:c r="H120" s="74"/>
+      <x:c r="I120" s="76"/>
+      <x:c r="J120" s="64"/>
+      <x:c r="K120" s="76"/>
+      <x:c r="L120" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="121" ht="22" customHeight="1">
       <x:c r="A121" s="21" t="str">
@@ -2074,8 +3001,14 @@
       <x:c r="D121" s="21"/>
       <x:c r="E121" s="21"/>
       <x:c r="F121" s="22"/>
-      <x:c r="G121" s="23"/>
-      <x:c r="H121" s="24"/>
+      <x:c r="G121" s="73"/>
+      <x:c r="H121" s="74"/>
+      <x:c r="I121" s="76"/>
+      <x:c r="J121" s="64"/>
+      <x:c r="K121" s="76"/>
+      <x:c r="L121" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="122" ht="22" customHeight="1">
       <x:c r="A122" s="21" t="str">
@@ -2086,8 +3019,14 @@
       <x:c r="D122" s="21"/>
       <x:c r="E122" s="21"/>
       <x:c r="F122" s="22"/>
-      <x:c r="G122" s="23"/>
-      <x:c r="H122" s="24"/>
+      <x:c r="G122" s="73"/>
+      <x:c r="H122" s="74"/>
+      <x:c r="I122" s="76"/>
+      <x:c r="J122" s="64"/>
+      <x:c r="K122" s="76"/>
+      <x:c r="L122" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="123" ht="22" customHeight="1">
       <x:c r="A123" s="21" t="str">
@@ -2098,8 +3037,14 @@
       <x:c r="D123" s="21"/>
       <x:c r="E123" s="21"/>
       <x:c r="F123" s="22"/>
-      <x:c r="G123" s="23"/>
-      <x:c r="H123" s="24"/>
+      <x:c r="G123" s="73"/>
+      <x:c r="H123" s="74"/>
+      <x:c r="I123" s="76"/>
+      <x:c r="J123" s="64"/>
+      <x:c r="K123" s="76"/>
+      <x:c r="L123" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="124" ht="22" customHeight="1">
       <x:c r="A124" s="21" t="str">
@@ -2110,8 +3055,14 @@
       <x:c r="D124" s="21"/>
       <x:c r="E124" s="21"/>
       <x:c r="F124" s="22"/>
-      <x:c r="G124" s="23"/>
-      <x:c r="H124" s="24"/>
+      <x:c r="G124" s="73"/>
+      <x:c r="H124" s="74"/>
+      <x:c r="I124" s="76"/>
+      <x:c r="J124" s="64"/>
+      <x:c r="K124" s="76"/>
+      <x:c r="L124" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="125" ht="22" customHeight="1">
       <x:c r="A125" s="21" t="str">
@@ -2122,8 +3073,14 @@
       <x:c r="D125" s="21"/>
       <x:c r="E125" s="21"/>
       <x:c r="F125" s="22"/>
-      <x:c r="G125" s="23"/>
-      <x:c r="H125" s="24"/>
+      <x:c r="G125" s="73"/>
+      <x:c r="H125" s="74"/>
+      <x:c r="I125" s="76"/>
+      <x:c r="J125" s="64"/>
+      <x:c r="K125" s="76"/>
+      <x:c r="L125" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="126" ht="22" customHeight="1">
       <x:c r="A126" s="21" t="str">
@@ -2134,8 +3091,14 @@
       <x:c r="D126" s="21"/>
       <x:c r="E126" s="21"/>
       <x:c r="F126" s="22"/>
-      <x:c r="G126" s="23"/>
-      <x:c r="H126" s="24"/>
+      <x:c r="G126" s="73"/>
+      <x:c r="H126" s="74"/>
+      <x:c r="I126" s="76"/>
+      <x:c r="J126" s="64"/>
+      <x:c r="K126" s="76"/>
+      <x:c r="L126" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="127" ht="22" customHeight="1">
       <x:c r="A127" s="21" t="str">
@@ -2146,8 +3109,14 @@
       <x:c r="D127" s="21"/>
       <x:c r="E127" s="21"/>
       <x:c r="F127" s="22"/>
-      <x:c r="G127" s="23"/>
-      <x:c r="H127" s="24"/>
+      <x:c r="G127" s="73"/>
+      <x:c r="H127" s="74"/>
+      <x:c r="I127" s="76"/>
+      <x:c r="J127" s="64"/>
+      <x:c r="K127" s="76"/>
+      <x:c r="L127" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="128" ht="22" customHeight="1">
       <x:c r="A128" s="21" t="str">
@@ -2158,8 +3127,14 @@
       <x:c r="D128" s="21"/>
       <x:c r="E128" s="21"/>
       <x:c r="F128" s="22"/>
-      <x:c r="G128" s="23"/>
-      <x:c r="H128" s="24"/>
+      <x:c r="G128" s="73"/>
+      <x:c r="H128" s="74"/>
+      <x:c r="I128" s="76"/>
+      <x:c r="J128" s="64"/>
+      <x:c r="K128" s="76"/>
+      <x:c r="L128" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="129" ht="22" customHeight="1">
       <x:c r="A129" s="21" t="str">
@@ -2170,8 +3145,14 @@
       <x:c r="D129" s="21"/>
       <x:c r="E129" s="21"/>
       <x:c r="F129" s="22"/>
-      <x:c r="G129" s="23"/>
-      <x:c r="H129" s="24"/>
+      <x:c r="G129" s="73"/>
+      <x:c r="H129" s="74"/>
+      <x:c r="I129" s="76"/>
+      <x:c r="J129" s="64"/>
+      <x:c r="K129" s="76"/>
+      <x:c r="L129" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="130" ht="22" customHeight="1">
       <x:c r="A130" s="21" t="str">
@@ -2182,8 +3163,14 @@
       <x:c r="D130" s="21"/>
       <x:c r="E130" s="21"/>
       <x:c r="F130" s="22"/>
-      <x:c r="G130" s="23"/>
-      <x:c r="H130" s="24"/>
+      <x:c r="G130" s="73"/>
+      <x:c r="H130" s="74"/>
+      <x:c r="I130" s="76"/>
+      <x:c r="J130" s="64"/>
+      <x:c r="K130" s="76"/>
+      <x:c r="L130" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="131" ht="22" customHeight="1">
       <x:c r="A131" s="21" t="str">
@@ -2194,8 +3181,14 @@
       <x:c r="D131" s="21"/>
       <x:c r="E131" s="21"/>
       <x:c r="F131" s="22"/>
-      <x:c r="G131" s="23"/>
-      <x:c r="H131" s="24"/>
+      <x:c r="G131" s="73"/>
+      <x:c r="H131" s="74"/>
+      <x:c r="I131" s="76"/>
+      <x:c r="J131" s="64"/>
+      <x:c r="K131" s="76"/>
+      <x:c r="L131" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="132" ht="22" customHeight="1">
       <x:c r="A132" s="21" t="str">
@@ -2206,8 +3199,14 @@
       <x:c r="D132" s="21"/>
       <x:c r="E132" s="21"/>
       <x:c r="F132" s="22"/>
-      <x:c r="G132" s="23"/>
-      <x:c r="H132" s="24"/>
+      <x:c r="G132" s="73"/>
+      <x:c r="H132" s="74"/>
+      <x:c r="I132" s="76"/>
+      <x:c r="J132" s="64"/>
+      <x:c r="K132" s="76"/>
+      <x:c r="L132" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="133" ht="22" customHeight="1">
       <x:c r="A133" s="21" t="str">
@@ -2218,8 +3217,14 @@
       <x:c r="D133" s="21"/>
       <x:c r="E133" s="21"/>
       <x:c r="F133" s="22"/>
-      <x:c r="G133" s="23"/>
-      <x:c r="H133" s="24"/>
+      <x:c r="G133" s="73"/>
+      <x:c r="H133" s="74"/>
+      <x:c r="I133" s="76"/>
+      <x:c r="J133" s="64"/>
+      <x:c r="K133" s="76"/>
+      <x:c r="L133" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="134" ht="22" customHeight="1">
       <x:c r="A134" s="21" t="str">
@@ -2230,8 +3235,14 @@
       <x:c r="D134" s="21"/>
       <x:c r="E134" s="21"/>
       <x:c r="F134" s="22"/>
-      <x:c r="G134" s="23"/>
-      <x:c r="H134" s="24"/>
+      <x:c r="G134" s="73"/>
+      <x:c r="H134" s="74"/>
+      <x:c r="I134" s="76"/>
+      <x:c r="J134" s="64"/>
+      <x:c r="K134" s="76"/>
+      <x:c r="L134" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="135" ht="22" customHeight="1">
       <x:c r="A135" s="21" t="str">
@@ -2242,8 +3253,14 @@
       <x:c r="D135" s="21"/>
       <x:c r="E135" s="21"/>
       <x:c r="F135" s="22"/>
-      <x:c r="G135" s="23"/>
-      <x:c r="H135" s="24"/>
+      <x:c r="G135" s="73"/>
+      <x:c r="H135" s="74"/>
+      <x:c r="I135" s="76"/>
+      <x:c r="J135" s="64"/>
+      <x:c r="K135" s="76"/>
+      <x:c r="L135" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="136" ht="22" customHeight="1">
       <x:c r="A136" s="21" t="str">
@@ -2254,8 +3271,14 @@
       <x:c r="D136" s="21"/>
       <x:c r="E136" s="21"/>
       <x:c r="F136" s="22"/>
-      <x:c r="G136" s="23"/>
-      <x:c r="H136" s="24"/>
+      <x:c r="G136" s="73"/>
+      <x:c r="H136" s="74"/>
+      <x:c r="I136" s="76"/>
+      <x:c r="J136" s="64"/>
+      <x:c r="K136" s="76"/>
+      <x:c r="L136" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="137" ht="22" customHeight="1">
       <x:c r="A137" s="21" t="str">
@@ -2266,8 +3289,14 @@
       <x:c r="D137" s="21"/>
       <x:c r="E137" s="21"/>
       <x:c r="F137" s="22"/>
-      <x:c r="G137" s="23"/>
-      <x:c r="H137" s="24"/>
+      <x:c r="G137" s="73"/>
+      <x:c r="H137" s="74"/>
+      <x:c r="I137" s="76"/>
+      <x:c r="J137" s="64"/>
+      <x:c r="K137" s="76"/>
+      <x:c r="L137" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="138" ht="22" customHeight="1">
       <x:c r="A138" s="21" t="str">
@@ -2278,8 +3307,14 @@
       <x:c r="D138" s="21"/>
       <x:c r="E138" s="21"/>
       <x:c r="F138" s="22"/>
-      <x:c r="G138" s="23"/>
-      <x:c r="H138" s="24"/>
+      <x:c r="G138" s="73"/>
+      <x:c r="H138" s="74"/>
+      <x:c r="I138" s="76"/>
+      <x:c r="J138" s="64"/>
+      <x:c r="K138" s="76"/>
+      <x:c r="L138" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="139" ht="22" customHeight="1">
       <x:c r="A139" s="21" t="str">
@@ -2290,8 +3325,14 @@
       <x:c r="D139" s="21"/>
       <x:c r="E139" s="21"/>
       <x:c r="F139" s="22"/>
-      <x:c r="G139" s="23"/>
-      <x:c r="H139" s="24"/>
+      <x:c r="G139" s="73"/>
+      <x:c r="H139" s="74"/>
+      <x:c r="I139" s="76"/>
+      <x:c r="J139" s="64"/>
+      <x:c r="K139" s="76"/>
+      <x:c r="L139" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="140" ht="22" customHeight="1">
       <x:c r="A140" s="21" t="str">
@@ -2302,8 +3343,14 @@
       <x:c r="D140" s="21"/>
       <x:c r="E140" s="21"/>
       <x:c r="F140" s="22"/>
-      <x:c r="G140" s="23"/>
-      <x:c r="H140" s="24"/>
+      <x:c r="G140" s="73"/>
+      <x:c r="H140" s="74"/>
+      <x:c r="I140" s="76"/>
+      <x:c r="J140" s="64"/>
+      <x:c r="K140" s="76"/>
+      <x:c r="L140" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="141" ht="22" customHeight="1">
       <x:c r="A141" s="21" t="str">
@@ -2314,8 +3361,14 @@
       <x:c r="D141" s="21"/>
       <x:c r="E141" s="21"/>
       <x:c r="F141" s="22"/>
-      <x:c r="G141" s="23"/>
-      <x:c r="H141" s="24"/>
+      <x:c r="G141" s="73"/>
+      <x:c r="H141" s="74"/>
+      <x:c r="I141" s="76"/>
+      <x:c r="J141" s="64"/>
+      <x:c r="K141" s="76"/>
+      <x:c r="L141" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="142" ht="22" customHeight="1">
       <x:c r="A142" s="21" t="str">
@@ -2326,8 +3379,14 @@
       <x:c r="D142" s="21"/>
       <x:c r="E142" s="21"/>
       <x:c r="F142" s="22"/>
-      <x:c r="G142" s="23"/>
-      <x:c r="H142" s="24"/>
+      <x:c r="G142" s="73"/>
+      <x:c r="H142" s="74"/>
+      <x:c r="I142" s="76"/>
+      <x:c r="J142" s="64"/>
+      <x:c r="K142" s="76"/>
+      <x:c r="L142" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="143" ht="22" customHeight="1">
       <x:c r="A143" s="21" t="str">
@@ -2338,8 +3397,14 @@
       <x:c r="D143" s="21"/>
       <x:c r="E143" s="21"/>
       <x:c r="F143" s="22"/>
-      <x:c r="G143" s="23"/>
-      <x:c r="H143" s="24"/>
+      <x:c r="G143" s="73"/>
+      <x:c r="H143" s="74"/>
+      <x:c r="I143" s="76"/>
+      <x:c r="J143" s="64"/>
+      <x:c r="K143" s="76"/>
+      <x:c r="L143" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="144" ht="22" customHeight="1">
       <x:c r="A144" s="21" t="str">
@@ -2350,8 +3415,14 @@
       <x:c r="D144" s="21"/>
       <x:c r="E144" s="21"/>
       <x:c r="F144" s="22"/>
-      <x:c r="G144" s="23"/>
-      <x:c r="H144" s="24"/>
+      <x:c r="G144" s="73"/>
+      <x:c r="H144" s="74"/>
+      <x:c r="I144" s="76"/>
+      <x:c r="J144" s="64"/>
+      <x:c r="K144" s="76"/>
+      <x:c r="L144" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="145" ht="22" customHeight="1">
       <x:c r="A145" s="21" t="str">
@@ -2362,8 +3433,14 @@
       <x:c r="D145" s="21"/>
       <x:c r="E145" s="21"/>
       <x:c r="F145" s="22"/>
-      <x:c r="G145" s="23"/>
-      <x:c r="H145" s="24"/>
+      <x:c r="G145" s="73"/>
+      <x:c r="H145" s="74"/>
+      <x:c r="I145" s="76"/>
+      <x:c r="J145" s="64"/>
+      <x:c r="K145" s="76"/>
+      <x:c r="L145" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="146" ht="22" customHeight="1">
       <x:c r="A146" s="21" t="str">
@@ -2374,8 +3451,14 @@
       <x:c r="D146" s="21"/>
       <x:c r="E146" s="21"/>
       <x:c r="F146" s="22"/>
-      <x:c r="G146" s="23"/>
-      <x:c r="H146" s="24"/>
+      <x:c r="G146" s="73"/>
+      <x:c r="H146" s="74"/>
+      <x:c r="I146" s="76"/>
+      <x:c r="J146" s="64"/>
+      <x:c r="K146" s="76"/>
+      <x:c r="L146" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="147" ht="22" customHeight="1">
       <x:c r="A147" s="21" t="str">
@@ -2386,8 +3469,14 @@
       <x:c r="D147" s="21"/>
       <x:c r="E147" s="21"/>
       <x:c r="F147" s="22"/>
-      <x:c r="G147" s="23"/>
-      <x:c r="H147" s="24"/>
+      <x:c r="G147" s="73"/>
+      <x:c r="H147" s="74"/>
+      <x:c r="I147" s="76"/>
+      <x:c r="J147" s="64"/>
+      <x:c r="K147" s="76"/>
+      <x:c r="L147" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="148" ht="22" customHeight="1">
       <x:c r="A148" s="21" t="str">
@@ -2398,8 +3487,14 @@
       <x:c r="D148" s="21"/>
       <x:c r="E148" s="21"/>
       <x:c r="F148" s="22"/>
-      <x:c r="G148" s="23"/>
-      <x:c r="H148" s="24"/>
+      <x:c r="G148" s="73"/>
+      <x:c r="H148" s="74"/>
+      <x:c r="I148" s="76"/>
+      <x:c r="J148" s="64"/>
+      <x:c r="K148" s="76"/>
+      <x:c r="L148" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="149" ht="22" customHeight="1">
       <x:c r="A149" s="21" t="str">
@@ -2410,8 +3505,14 @@
       <x:c r="D149" s="21"/>
       <x:c r="E149" s="21"/>
       <x:c r="F149" s="22"/>
-      <x:c r="G149" s="23"/>
-      <x:c r="H149" s="24"/>
+      <x:c r="G149" s="73"/>
+      <x:c r="H149" s="74"/>
+      <x:c r="I149" s="76"/>
+      <x:c r="J149" s="64"/>
+      <x:c r="K149" s="76"/>
+      <x:c r="L149" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="150" ht="22" customHeight="1">
       <x:c r="A150" s="21" t="str">
@@ -2422,8 +3523,14 @@
       <x:c r="D150" s="21"/>
       <x:c r="E150" s="21"/>
       <x:c r="F150" s="22"/>
-      <x:c r="G150" s="23"/>
-      <x:c r="H150" s="24"/>
+      <x:c r="G150" s="73"/>
+      <x:c r="H150" s="74"/>
+      <x:c r="I150" s="76"/>
+      <x:c r="J150" s="64"/>
+      <x:c r="K150" s="76"/>
+      <x:c r="L150" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="151" ht="22" customHeight="1">
       <x:c r="A151" s="21" t="str">
@@ -2434,8 +3541,14 @@
       <x:c r="D151" s="21"/>
       <x:c r="E151" s="21"/>
       <x:c r="F151" s="22"/>
-      <x:c r="G151" s="23"/>
-      <x:c r="H151" s="24"/>
+      <x:c r="G151" s="73"/>
+      <x:c r="H151" s="74"/>
+      <x:c r="I151" s="76"/>
+      <x:c r="J151" s="64"/>
+      <x:c r="K151" s="76"/>
+      <x:c r="L151" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="152" ht="22" customHeight="1">
       <x:c r="A152" s="21" t="str">
@@ -2446,8 +3559,14 @@
       <x:c r="D152" s="21"/>
       <x:c r="E152" s="21"/>
       <x:c r="F152" s="22"/>
-      <x:c r="G152" s="23"/>
-      <x:c r="H152" s="24"/>
+      <x:c r="G152" s="73"/>
+      <x:c r="H152" s="74"/>
+      <x:c r="I152" s="76"/>
+      <x:c r="J152" s="64"/>
+      <x:c r="K152" s="76"/>
+      <x:c r="L152" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="153" ht="22" customHeight="1">
       <x:c r="A153" s="21" t="str">
@@ -2458,8 +3577,14 @@
       <x:c r="D153" s="21"/>
       <x:c r="E153" s="21"/>
       <x:c r="F153" s="22"/>
-      <x:c r="G153" s="23"/>
-      <x:c r="H153" s="24"/>
+      <x:c r="G153" s="73"/>
+      <x:c r="H153" s="74"/>
+      <x:c r="I153" s="76"/>
+      <x:c r="J153" s="64"/>
+      <x:c r="K153" s="76"/>
+      <x:c r="L153" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="154" ht="22" customHeight="1">
       <x:c r="A154" s="21" t="str">
@@ -2470,8 +3595,14 @@
       <x:c r="D154" s="21"/>
       <x:c r="E154" s="21"/>
       <x:c r="F154" s="22"/>
-      <x:c r="G154" s="23"/>
-      <x:c r="H154" s="24"/>
+      <x:c r="G154" s="73"/>
+      <x:c r="H154" s="74"/>
+      <x:c r="I154" s="76"/>
+      <x:c r="J154" s="64"/>
+      <x:c r="K154" s="76"/>
+      <x:c r="L154" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="155" ht="22" customHeight="1">
       <x:c r="A155" s="21" t="str">
@@ -2482,8 +3613,14 @@
       <x:c r="D155" s="21"/>
       <x:c r="E155" s="21"/>
       <x:c r="F155" s="22"/>
-      <x:c r="G155" s="23"/>
-      <x:c r="H155" s="24"/>
+      <x:c r="G155" s="73"/>
+      <x:c r="H155" s="74"/>
+      <x:c r="I155" s="76"/>
+      <x:c r="J155" s="64"/>
+      <x:c r="K155" s="76"/>
+      <x:c r="L155" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="156" ht="22" customHeight="1">
       <x:c r="A156" s="21" t="str">
@@ -2494,8 +3631,14 @@
       <x:c r="D156" s="21"/>
       <x:c r="E156" s="21"/>
       <x:c r="F156" s="22"/>
-      <x:c r="G156" s="23"/>
-      <x:c r="H156" s="24"/>
+      <x:c r="G156" s="73"/>
+      <x:c r="H156" s="74"/>
+      <x:c r="I156" s="76"/>
+      <x:c r="J156" s="64"/>
+      <x:c r="K156" s="76"/>
+      <x:c r="L156" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="157" ht="22" customHeight="1">
       <x:c r="A157" s="21" t="str">
@@ -2506,8 +3649,14 @@
       <x:c r="D157" s="21"/>
       <x:c r="E157" s="21"/>
       <x:c r="F157" s="22"/>
-      <x:c r="G157" s="23"/>
-      <x:c r="H157" s="24"/>
+      <x:c r="G157" s="73"/>
+      <x:c r="H157" s="74"/>
+      <x:c r="I157" s="76"/>
+      <x:c r="J157" s="64"/>
+      <x:c r="K157" s="76"/>
+      <x:c r="L157" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="158" ht="22" customHeight="1">
       <x:c r="A158" s="21" t="str">
@@ -2518,8 +3667,14 @@
       <x:c r="D158" s="21"/>
       <x:c r="E158" s="21"/>
       <x:c r="F158" s="22"/>
-      <x:c r="G158" s="23"/>
-      <x:c r="H158" s="24"/>
+      <x:c r="G158" s="73"/>
+      <x:c r="H158" s="74"/>
+      <x:c r="I158" s="76"/>
+      <x:c r="J158" s="64"/>
+      <x:c r="K158" s="76"/>
+      <x:c r="L158" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="159" ht="22" customHeight="1">
       <x:c r="A159" s="21" t="str">
@@ -2530,8 +3685,14 @@
       <x:c r="D159" s="21"/>
       <x:c r="E159" s="21"/>
       <x:c r="F159" s="22"/>
-      <x:c r="G159" s="23"/>
-      <x:c r="H159" s="24"/>
+      <x:c r="G159" s="73"/>
+      <x:c r="H159" s="74"/>
+      <x:c r="I159" s="76"/>
+      <x:c r="J159" s="64"/>
+      <x:c r="K159" s="76"/>
+      <x:c r="L159" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="160" ht="22" customHeight="1">
       <x:c r="A160" s="21" t="str">
@@ -2542,8 +3703,14 @@
       <x:c r="D160" s="21"/>
       <x:c r="E160" s="21"/>
       <x:c r="F160" s="22"/>
-      <x:c r="G160" s="23"/>
-      <x:c r="H160" s="24"/>
+      <x:c r="G160" s="73"/>
+      <x:c r="H160" s="74"/>
+      <x:c r="I160" s="76"/>
+      <x:c r="J160" s="64"/>
+      <x:c r="K160" s="76"/>
+      <x:c r="L160" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="161" ht="22" customHeight="1">
       <x:c r="A161" s="21" t="str">
@@ -2554,8 +3721,14 @@
       <x:c r="D161" s="21"/>
       <x:c r="E161" s="21"/>
       <x:c r="F161" s="22"/>
-      <x:c r="G161" s="23"/>
-      <x:c r="H161" s="24"/>
+      <x:c r="G161" s="73"/>
+      <x:c r="H161" s="74"/>
+      <x:c r="I161" s="76"/>
+      <x:c r="J161" s="64"/>
+      <x:c r="K161" s="76"/>
+      <x:c r="L161" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="162" ht="22" customHeight="1">
       <x:c r="A162" s="21" t="str">
@@ -2566,8 +3739,14 @@
       <x:c r="D162" s="21"/>
       <x:c r="E162" s="21"/>
       <x:c r="F162" s="22"/>
-      <x:c r="G162" s="23"/>
-      <x:c r="H162" s="24"/>
+      <x:c r="G162" s="73"/>
+      <x:c r="H162" s="74"/>
+      <x:c r="I162" s="76"/>
+      <x:c r="J162" s="64"/>
+      <x:c r="K162" s="76"/>
+      <x:c r="L162" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="163" ht="22" customHeight="1">
       <x:c r="A163" s="21" t="str">
@@ -2578,8 +3757,14 @@
       <x:c r="D163" s="21"/>
       <x:c r="E163" s="21"/>
       <x:c r="F163" s="22"/>
-      <x:c r="G163" s="23"/>
-      <x:c r="H163" s="24"/>
+      <x:c r="G163" s="73"/>
+      <x:c r="H163" s="74"/>
+      <x:c r="I163" s="76"/>
+      <x:c r="J163" s="64"/>
+      <x:c r="K163" s="76"/>
+      <x:c r="L163" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="164" ht="22" customHeight="1">
       <x:c r="A164" s="21" t="str">
@@ -2590,8 +3775,14 @@
       <x:c r="D164" s="21"/>
       <x:c r="E164" s="21"/>
       <x:c r="F164" s="22"/>
-      <x:c r="G164" s="23"/>
-      <x:c r="H164" s="24"/>
+      <x:c r="G164" s="73"/>
+      <x:c r="H164" s="74"/>
+      <x:c r="I164" s="76"/>
+      <x:c r="J164" s="64"/>
+      <x:c r="K164" s="76"/>
+      <x:c r="L164" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="165" ht="22" customHeight="1">
       <x:c r="A165" s="21" t="str">
@@ -2602,8 +3793,14 @@
       <x:c r="D165" s="21"/>
       <x:c r="E165" s="21"/>
       <x:c r="F165" s="22"/>
-      <x:c r="G165" s="23"/>
-      <x:c r="H165" s="24"/>
+      <x:c r="G165" s="73"/>
+      <x:c r="H165" s="74"/>
+      <x:c r="I165" s="76"/>
+      <x:c r="J165" s="64"/>
+      <x:c r="K165" s="76"/>
+      <x:c r="L165" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="166" ht="22" customHeight="1">
       <x:c r="A166" s="21" t="str">
@@ -2614,8 +3811,14 @@
       <x:c r="D166" s="21"/>
       <x:c r="E166" s="21"/>
       <x:c r="F166" s="22"/>
-      <x:c r="G166" s="23"/>
-      <x:c r="H166" s="24"/>
+      <x:c r="G166" s="73"/>
+      <x:c r="H166" s="74"/>
+      <x:c r="I166" s="76"/>
+      <x:c r="J166" s="64"/>
+      <x:c r="K166" s="76"/>
+      <x:c r="L166" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="167" ht="22" customHeight="1">
       <x:c r="A167" s="21" t="str">
@@ -2626,8 +3829,14 @@
       <x:c r="D167" s="21"/>
       <x:c r="E167" s="21"/>
       <x:c r="F167" s="22"/>
-      <x:c r="G167" s="23"/>
-      <x:c r="H167" s="24"/>
+      <x:c r="G167" s="73"/>
+      <x:c r="H167" s="74"/>
+      <x:c r="I167" s="76"/>
+      <x:c r="J167" s="64"/>
+      <x:c r="K167" s="76"/>
+      <x:c r="L167" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="168" ht="22" customHeight="1">
       <x:c r="A168" s="21" t="str">
@@ -2638,8 +3847,14 @@
       <x:c r="D168" s="21"/>
       <x:c r="E168" s="21"/>
       <x:c r="F168" s="22"/>
-      <x:c r="G168" s="23"/>
-      <x:c r="H168" s="24"/>
+      <x:c r="G168" s="73"/>
+      <x:c r="H168" s="74"/>
+      <x:c r="I168" s="76"/>
+      <x:c r="J168" s="64"/>
+      <x:c r="K168" s="76"/>
+      <x:c r="L168" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="169" ht="22" customHeight="1">
       <x:c r="A169" s="21" t="str">
@@ -2650,8 +3865,14 @@
       <x:c r="D169" s="21"/>
       <x:c r="E169" s="21"/>
       <x:c r="F169" s="22"/>
-      <x:c r="G169" s="23"/>
-      <x:c r="H169" s="24"/>
+      <x:c r="G169" s="73"/>
+      <x:c r="H169" s="74"/>
+      <x:c r="I169" s="76"/>
+      <x:c r="J169" s="64"/>
+      <x:c r="K169" s="76"/>
+      <x:c r="L169" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="170" ht="22" customHeight="1">
       <x:c r="A170" s="21" t="str">
@@ -2662,8 +3883,14 @@
       <x:c r="D170" s="21"/>
       <x:c r="E170" s="21"/>
       <x:c r="F170" s="22"/>
-      <x:c r="G170" s="23"/>
-      <x:c r="H170" s="24"/>
+      <x:c r="G170" s="73"/>
+      <x:c r="H170" s="74"/>
+      <x:c r="I170" s="76"/>
+      <x:c r="J170" s="64"/>
+      <x:c r="K170" s="76"/>
+      <x:c r="L170" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="171" ht="22" customHeight="1">
       <x:c r="A171" s="21" t="str">
@@ -2674,8 +3901,14 @@
       <x:c r="D171" s="21"/>
       <x:c r="E171" s="21"/>
       <x:c r="F171" s="22"/>
-      <x:c r="G171" s="23"/>
-      <x:c r="H171" s="24"/>
+      <x:c r="G171" s="73"/>
+      <x:c r="H171" s="74"/>
+      <x:c r="I171" s="76"/>
+      <x:c r="J171" s="64"/>
+      <x:c r="K171" s="76"/>
+      <x:c r="L171" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="172" ht="22" customHeight="1">
       <x:c r="A172" s="21" t="str">
@@ -2686,8 +3919,14 @@
       <x:c r="D172" s="21"/>
       <x:c r="E172" s="21"/>
       <x:c r="F172" s="22"/>
-      <x:c r="G172" s="23"/>
-      <x:c r="H172" s="24"/>
+      <x:c r="G172" s="73"/>
+      <x:c r="H172" s="74"/>
+      <x:c r="I172" s="76"/>
+      <x:c r="J172" s="64"/>
+      <x:c r="K172" s="76"/>
+      <x:c r="L172" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="173" ht="22" customHeight="1">
       <x:c r="A173" s="21" t="str">
@@ -2698,8 +3937,14 @@
       <x:c r="D173" s="21"/>
       <x:c r="E173" s="21"/>
       <x:c r="F173" s="22"/>
-      <x:c r="G173" s="23"/>
-      <x:c r="H173" s="24"/>
+      <x:c r="G173" s="73"/>
+      <x:c r="H173" s="74"/>
+      <x:c r="I173" s="76"/>
+      <x:c r="J173" s="64"/>
+      <x:c r="K173" s="76"/>
+      <x:c r="L173" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="174" ht="22" customHeight="1">
       <x:c r="A174" s="21" t="str">
@@ -2710,8 +3955,14 @@
       <x:c r="D174" s="21"/>
       <x:c r="E174" s="21"/>
       <x:c r="F174" s="22"/>
-      <x:c r="G174" s="23"/>
-      <x:c r="H174" s="24"/>
+      <x:c r="G174" s="73"/>
+      <x:c r="H174" s="74"/>
+      <x:c r="I174" s="76"/>
+      <x:c r="J174" s="64"/>
+      <x:c r="K174" s="76"/>
+      <x:c r="L174" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="175" ht="22" customHeight="1">
       <x:c r="A175" s="21" t="str">
@@ -2722,8 +3973,14 @@
       <x:c r="D175" s="21"/>
       <x:c r="E175" s="21"/>
       <x:c r="F175" s="22"/>
-      <x:c r="G175" s="23"/>
-      <x:c r="H175" s="24"/>
+      <x:c r="G175" s="73"/>
+      <x:c r="H175" s="74"/>
+      <x:c r="I175" s="76"/>
+      <x:c r="J175" s="64"/>
+      <x:c r="K175" s="76"/>
+      <x:c r="L175" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="176" ht="22" customHeight="1">
       <x:c r="A176" s="21" t="str">
@@ -2734,8 +3991,14 @@
       <x:c r="D176" s="21"/>
       <x:c r="E176" s="21"/>
       <x:c r="F176" s="22"/>
-      <x:c r="G176" s="23"/>
-      <x:c r="H176" s="24"/>
+      <x:c r="G176" s="73"/>
+      <x:c r="H176" s="74"/>
+      <x:c r="I176" s="76"/>
+      <x:c r="J176" s="64"/>
+      <x:c r="K176" s="76"/>
+      <x:c r="L176" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="177" ht="22" customHeight="1">
       <x:c r="A177" s="21" t="str">
@@ -2746,8 +4009,14 @@
       <x:c r="D177" s="21"/>
       <x:c r="E177" s="21"/>
       <x:c r="F177" s="22"/>
-      <x:c r="G177" s="23"/>
-      <x:c r="H177" s="24"/>
+      <x:c r="G177" s="73"/>
+      <x:c r="H177" s="74"/>
+      <x:c r="I177" s="76"/>
+      <x:c r="J177" s="64"/>
+      <x:c r="K177" s="76"/>
+      <x:c r="L177" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="178" ht="22" customHeight="1">
       <x:c r="A178" s="21" t="str">
@@ -2758,8 +4027,14 @@
       <x:c r="D178" s="21"/>
       <x:c r="E178" s="21"/>
       <x:c r="F178" s="22"/>
-      <x:c r="G178" s="23"/>
-      <x:c r="H178" s="24"/>
+      <x:c r="G178" s="73"/>
+      <x:c r="H178" s="74"/>
+      <x:c r="I178" s="76"/>
+      <x:c r="J178" s="64"/>
+      <x:c r="K178" s="76"/>
+      <x:c r="L178" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="179" ht="22" customHeight="1">
       <x:c r="A179" s="21" t="str">
@@ -2770,8 +4045,14 @@
       <x:c r="D179" s="21"/>
       <x:c r="E179" s="21"/>
       <x:c r="F179" s="22"/>
-      <x:c r="G179" s="23"/>
-      <x:c r="H179" s="24"/>
+      <x:c r="G179" s="73"/>
+      <x:c r="H179" s="74"/>
+      <x:c r="I179" s="76"/>
+      <x:c r="J179" s="64"/>
+      <x:c r="K179" s="76"/>
+      <x:c r="L179" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="180" ht="22" customHeight="1">
       <x:c r="A180" s="21" t="str">
@@ -2782,8 +4063,14 @@
       <x:c r="D180" s="21"/>
       <x:c r="E180" s="21"/>
       <x:c r="F180" s="22"/>
-      <x:c r="G180" s="23"/>
-      <x:c r="H180" s="24"/>
+      <x:c r="G180" s="73"/>
+      <x:c r="H180" s="74"/>
+      <x:c r="I180" s="76"/>
+      <x:c r="J180" s="64"/>
+      <x:c r="K180" s="76"/>
+      <x:c r="L180" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="181" ht="22" customHeight="1">
       <x:c r="A181" s="21" t="str">
@@ -2794,8 +4081,14 @@
       <x:c r="D181" s="21"/>
       <x:c r="E181" s="21"/>
       <x:c r="F181" s="22"/>
-      <x:c r="G181" s="23"/>
-      <x:c r="H181" s="24"/>
+      <x:c r="G181" s="73"/>
+      <x:c r="H181" s="74"/>
+      <x:c r="I181" s="76"/>
+      <x:c r="J181" s="64"/>
+      <x:c r="K181" s="76"/>
+      <x:c r="L181" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="182" ht="22" customHeight="1">
       <x:c r="A182" s="21" t="str">
@@ -2806,8 +4099,14 @@
       <x:c r="D182" s="21"/>
       <x:c r="E182" s="21"/>
       <x:c r="F182" s="22"/>
-      <x:c r="G182" s="23"/>
-      <x:c r="H182" s="24"/>
+      <x:c r="G182" s="73"/>
+      <x:c r="H182" s="74"/>
+      <x:c r="I182" s="76"/>
+      <x:c r="J182" s="64"/>
+      <x:c r="K182" s="76"/>
+      <x:c r="L182" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="183" ht="22" customHeight="1">
       <x:c r="A183" s="21" t="str">
@@ -2818,8 +4117,14 @@
       <x:c r="D183" s="21"/>
       <x:c r="E183" s="21"/>
       <x:c r="F183" s="22"/>
-      <x:c r="G183" s="23"/>
-      <x:c r="H183" s="24"/>
+      <x:c r="G183" s="73"/>
+      <x:c r="H183" s="74"/>
+      <x:c r="I183" s="76"/>
+      <x:c r="J183" s="64"/>
+      <x:c r="K183" s="76"/>
+      <x:c r="L183" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="184" ht="22" customHeight="1">
       <x:c r="A184" s="21" t="str">
@@ -2830,8 +4135,14 @@
       <x:c r="D184" s="21"/>
       <x:c r="E184" s="21"/>
       <x:c r="F184" s="22"/>
-      <x:c r="G184" s="23"/>
-      <x:c r="H184" s="24"/>
+      <x:c r="G184" s="73"/>
+      <x:c r="H184" s="74"/>
+      <x:c r="I184" s="76"/>
+      <x:c r="J184" s="64"/>
+      <x:c r="K184" s="76"/>
+      <x:c r="L184" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="185" ht="22" customHeight="1">
       <x:c r="A185" s="21" t="str">
@@ -2842,8 +4153,14 @@
       <x:c r="D185" s="21"/>
       <x:c r="E185" s="21"/>
       <x:c r="F185" s="22"/>
-      <x:c r="G185" s="23"/>
-      <x:c r="H185" s="24"/>
+      <x:c r="G185" s="73"/>
+      <x:c r="H185" s="74"/>
+      <x:c r="I185" s="76"/>
+      <x:c r="J185" s="64"/>
+      <x:c r="K185" s="76"/>
+      <x:c r="L185" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="186" ht="22" customHeight="1">
       <x:c r="A186" s="21" t="str">
@@ -2854,8 +4171,14 @@
       <x:c r="D186" s="21"/>
       <x:c r="E186" s="21"/>
       <x:c r="F186" s="22"/>
-      <x:c r="G186" s="23"/>
-      <x:c r="H186" s="24"/>
+      <x:c r="G186" s="73"/>
+      <x:c r="H186" s="74"/>
+      <x:c r="I186" s="76"/>
+      <x:c r="J186" s="64"/>
+      <x:c r="K186" s="76"/>
+      <x:c r="L186" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="187" ht="22" customHeight="1">
       <x:c r="A187" s="21" t="str">
@@ -2866,8 +4189,14 @@
       <x:c r="D187" s="21"/>
       <x:c r="E187" s="21"/>
       <x:c r="F187" s="22"/>
-      <x:c r="G187" s="23"/>
-      <x:c r="H187" s="24"/>
+      <x:c r="G187" s="73"/>
+      <x:c r="H187" s="74"/>
+      <x:c r="I187" s="76"/>
+      <x:c r="J187" s="64"/>
+      <x:c r="K187" s="76"/>
+      <x:c r="L187" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="188" ht="22" customHeight="1">
       <x:c r="A188" s="21" t="str">
@@ -2878,8 +4207,14 @@
       <x:c r="D188" s="21"/>
       <x:c r="E188" s="21"/>
       <x:c r="F188" s="22"/>
-      <x:c r="G188" s="23"/>
-      <x:c r="H188" s="24"/>
+      <x:c r="G188" s="73"/>
+      <x:c r="H188" s="74"/>
+      <x:c r="I188" s="76"/>
+      <x:c r="J188" s="64"/>
+      <x:c r="K188" s="76"/>
+      <x:c r="L188" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="189" ht="22" customHeight="1">
       <x:c r="A189" s="21" t="str">
@@ -2890,8 +4225,14 @@
       <x:c r="D189" s="21"/>
       <x:c r="E189" s="21"/>
       <x:c r="F189" s="22"/>
-      <x:c r="G189" s="23"/>
-      <x:c r="H189" s="24"/>
+      <x:c r="G189" s="73"/>
+      <x:c r="H189" s="74"/>
+      <x:c r="I189" s="76"/>
+      <x:c r="J189" s="64"/>
+      <x:c r="K189" s="76"/>
+      <x:c r="L189" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="190" ht="22" customHeight="1">
       <x:c r="A190" s="21" t="str">
@@ -2902,8 +4243,14 @@
       <x:c r="D190" s="21"/>
       <x:c r="E190" s="21"/>
       <x:c r="F190" s="22"/>
-      <x:c r="G190" s="23"/>
-      <x:c r="H190" s="24"/>
+      <x:c r="G190" s="73"/>
+      <x:c r="H190" s="74"/>
+      <x:c r="I190" s="76"/>
+      <x:c r="J190" s="64"/>
+      <x:c r="K190" s="76"/>
+      <x:c r="L190" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="191" ht="22" customHeight="1">
       <x:c r="A191" s="21" t="str">
@@ -2914,8 +4261,14 @@
       <x:c r="D191" s="21"/>
       <x:c r="E191" s="21"/>
       <x:c r="F191" s="22"/>
-      <x:c r="G191" s="23"/>
-      <x:c r="H191" s="24"/>
+      <x:c r="G191" s="73"/>
+      <x:c r="H191" s="74"/>
+      <x:c r="I191" s="76"/>
+      <x:c r="J191" s="64"/>
+      <x:c r="K191" s="76"/>
+      <x:c r="L191" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="192" ht="22" customHeight="1">
       <x:c r="A192" s="21" t="str">
@@ -2926,8 +4279,14 @@
       <x:c r="D192" s="21"/>
       <x:c r="E192" s="21"/>
       <x:c r="F192" s="22"/>
-      <x:c r="G192" s="23"/>
-      <x:c r="H192" s="24"/>
+      <x:c r="G192" s="73"/>
+      <x:c r="H192" s="74"/>
+      <x:c r="I192" s="76"/>
+      <x:c r="J192" s="64"/>
+      <x:c r="K192" s="76"/>
+      <x:c r="L192" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="193" ht="22" customHeight="1">
       <x:c r="A193" s="21" t="str">
@@ -2938,8 +4297,14 @@
       <x:c r="D193" s="21"/>
       <x:c r="E193" s="21"/>
       <x:c r="F193" s="22"/>
-      <x:c r="G193" s="23"/>
-      <x:c r="H193" s="24"/>
+      <x:c r="G193" s="73"/>
+      <x:c r="H193" s="74"/>
+      <x:c r="I193" s="76"/>
+      <x:c r="J193" s="64"/>
+      <x:c r="K193" s="76"/>
+      <x:c r="L193" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="194" ht="22" customHeight="1">
       <x:c r="A194" s="21" t="str">
@@ -2950,8 +4315,14 @@
       <x:c r="D194" s="21"/>
       <x:c r="E194" s="21"/>
       <x:c r="F194" s="22"/>
-      <x:c r="G194" s="23"/>
-      <x:c r="H194" s="24"/>
+      <x:c r="G194" s="73"/>
+      <x:c r="H194" s="74"/>
+      <x:c r="I194" s="76"/>
+      <x:c r="J194" s="64"/>
+      <x:c r="K194" s="76"/>
+      <x:c r="L194" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="195" ht="22" customHeight="1">
       <x:c r="A195" s="21" t="str">
@@ -2962,8 +4333,14 @@
       <x:c r="D195" s="21"/>
       <x:c r="E195" s="21"/>
       <x:c r="F195" s="22"/>
-      <x:c r="G195" s="23"/>
-      <x:c r="H195" s="24"/>
+      <x:c r="G195" s="73"/>
+      <x:c r="H195" s="74"/>
+      <x:c r="I195" s="76"/>
+      <x:c r="J195" s="64"/>
+      <x:c r="K195" s="76"/>
+      <x:c r="L195" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="196" ht="22" customHeight="1">
       <x:c r="A196" s="21" t="str">
@@ -2974,8 +4351,14 @@
       <x:c r="D196" s="21"/>
       <x:c r="E196" s="21"/>
       <x:c r="F196" s="22"/>
-      <x:c r="G196" s="23"/>
-      <x:c r="H196" s="24"/>
+      <x:c r="G196" s="73"/>
+      <x:c r="H196" s="74"/>
+      <x:c r="I196" s="76"/>
+      <x:c r="J196" s="64"/>
+      <x:c r="K196" s="76"/>
+      <x:c r="L196" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="197" ht="22" customHeight="1">
       <x:c r="A197" s="21" t="str">
@@ -2986,8 +4369,14 @@
       <x:c r="D197" s="21"/>
       <x:c r="E197" s="21"/>
       <x:c r="F197" s="22"/>
-      <x:c r="G197" s="23"/>
-      <x:c r="H197" s="24"/>
+      <x:c r="G197" s="73"/>
+      <x:c r="H197" s="74"/>
+      <x:c r="I197" s="76"/>
+      <x:c r="J197" s="64"/>
+      <x:c r="K197" s="76"/>
+      <x:c r="L197" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="198" ht="22" customHeight="1">
       <x:c r="A198" s="21" t="str">
@@ -2998,8 +4387,14 @@
       <x:c r="D198" s="21"/>
       <x:c r="E198" s="21"/>
       <x:c r="F198" s="22"/>
-      <x:c r="G198" s="23"/>
-      <x:c r="H198" s="24"/>
+      <x:c r="G198" s="73"/>
+      <x:c r="H198" s="74"/>
+      <x:c r="I198" s="76"/>
+      <x:c r="J198" s="64"/>
+      <x:c r="K198" s="76"/>
+      <x:c r="L198" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="199" ht="22" customHeight="1">
       <x:c r="A199" s="21" t="str">
@@ -3010,8 +4405,14 @@
       <x:c r="D199" s="21"/>
       <x:c r="E199" s="21"/>
       <x:c r="F199" s="22"/>
-      <x:c r="G199" s="23"/>
-      <x:c r="H199" s="24"/>
+      <x:c r="G199" s="73"/>
+      <x:c r="H199" s="74"/>
+      <x:c r="I199" s="76"/>
+      <x:c r="J199" s="64"/>
+      <x:c r="K199" s="76"/>
+      <x:c r="L199" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="200" ht="22" customHeight="1">
       <x:c r="A200" s="21" t="str">
@@ -3022,8 +4423,14 @@
       <x:c r="D200" s="21"/>
       <x:c r="E200" s="21"/>
       <x:c r="F200" s="22"/>
-      <x:c r="G200" s="23"/>
-      <x:c r="H200" s="24"/>
+      <x:c r="G200" s="73"/>
+      <x:c r="H200" s="74"/>
+      <x:c r="I200" s="76"/>
+      <x:c r="J200" s="64"/>
+      <x:c r="K200" s="76"/>
+      <x:c r="L200" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="201" ht="22" customHeight="1">
       <x:c r="A201" s="21" t="str">
@@ -3034,14 +4441,45 @@
       <x:c r="D201" s="21"/>
       <x:c r="E201" s="21"/>
       <x:c r="F201" s="22"/>
-      <x:c r="G201" s="23"/>
-      <x:c r="H201" s="24"/>
+      <x:c r="G201" s="73"/>
+      <x:c r="H201" s="74"/>
+      <x:c r="I201" s="76"/>
+      <x:c r="J201" s="64"/>
+      <x:c r="K201" s="76"/>
+      <x:c r="L201" s="65" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
+  <x:conditionalFormatting sqref="G2:G201">
+    <x:cfRule type="expression" dxfId="0" priority="1">
+      <x:formula>AND($C2&lt;&gt;"",LEN(TRIM(G2&amp;""))=0)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="H2:H201">
+    <x:cfRule type="expression" dxfId="1" priority="2">
+      <x:formula>AND($C2&lt;&gt;"",LEN(TRIM(H2&amp;""))=0)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="I2:I201">
+    <x:cfRule type="expression" dxfId="2" priority="3">
+      <x:formula>AND($C2&lt;&gt;"",LEN(TRIM(I2&amp;""))=0)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="K2:K201">
+    <x:cfRule type="expression" dxfId="3" priority="4">
+      <x:formula>AND($C2&lt;&gt;"",LEN(TRIM(K2&amp;""))=0)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="L2:L201">
+      <x:formula1>"No,Yes"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50b48d533a814bc6"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb25c9d8a583047ab"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0a0672dd6fc48a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c19c783324945ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3133,10 +4571,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B8" s="37" t="str">
-        <x:v>保存后上传到 Create RFQ</x:v>
+        <x:v>保存、上传，核对预览后确认运行</x:v>
       </x:c>
       <x:c r="C8" s="37" t="str">
-        <x:v>Save, upload, validate, then run Create RFQ</x:v>
+        <x:v>Save, upload, review and confirm Production</x:v>
       </x:c>
       <x:c r="D8" s="37"/>
       <x:c r="E8" s="37"/>
@@ -3192,7 +4630,7 @@
         <x:v>C100</x:v>
       </x:c>
       <x:c r="E13" s="42" t="str">
-        <x:v>测试 / Test</x:v>
+        <x:v>测试（开发）/ Dev QA</x:v>
       </x:c>
       <x:c r="F13" s="42" t="str">
         <x:v>CEQ QA [321]</x:v>
@@ -3242,9 +4680,9 @@
       <x:c r="G15"/>
       <x:c r="H15"/>
     </x:row>
-    <x:row r="16" ht="38" customHeight="1">
+    <x:row r="16" ht="66" customHeight="1">
       <x:c r="A16" s="42" t="str">
-        <x:v>Intended Supplier</x:v>
+        <x:v>Supplier Parma</x:v>
       </x:c>
       <x:c r="B16" s="42" t="str">
         <x:v>目标供应商 Parma 号</x:v>
@@ -3256,7 +4694,8 @@
         <x:v>提醒 / Note</x:v>
       </x:c>
       <x:c r="F16" s="46" t="str">
-        <x:v>请先在测试系统验证。正式系统会创建真实业务数据。</x:v>
+        <x:v>应用默认正式系统；请核对预览后确认。
+Production: review and confirm.</x:v>
       </x:c>
       <x:c r="G16" s="46"/>
       <x:c r="H16" s="46"/>
@@ -3282,23 +4721,100 @@
       <x:c r="C18" s="42" t="str">
         <x:v>2026-12-31</x:v>
       </x:c>
-    </x:row>
-    <x:row r="19" ht="24" customHeight="1">
-      <x:c r="A19" s="42" t="str">
+      <x:c r="E18" s="47" t="str">
+        <x:v>同 Plant + Project + Parma 合并；每个 RFQ 最多 50 个物料。
+Same Plant + Project + Parma; max 50 materials per RFQ.</x:v>
+      </x:c>
+      <x:c r="F18" s="47"/>
+      <x:c r="G18" s="47"/>
+      <x:c r="H18" s="47"/>
+    </x:row>
+    <x:row r="19" ht="42" customHeight="1">
+      <x:c r="A19" s="71" t="str">
         <x:v>PPAP Date / Technology</x:v>
       </x:c>
-      <x:c r="B19" s="42" t="str">
-        <x:v>可选字段</x:v>
-      </x:c>
-      <x:c r="C19" s="42" t="str">
-        <x:v>可留空</x:v>
-      </x:c>
+      <x:c r="B19" s="71" t="str">
+        <x:v>G / H 必填。PPAP 日期 YYYY-MM-DD</x:v>
+      </x:c>
+      <x:c r="C19" s="71" t="str">
+        <x:v>2026-12-31 / 技术负责人</x:v>
+      </x:c>
+      <x:c r="E19" s="47"/>
+      <x:c r="F19" s="47"/>
+      <x:c r="G19" s="47"/>
+      <x:c r="H19" s="47"/>
+    </x:row>
+    <x:row r="21" ht="46" customHeight="1">
+      <x:c r="A21" s="61" t="str">
+        <x:v>12 MR Qty</x:v>
+      </x:c>
+      <x:c r="B21" s="61" t="str">
+        <x:v>I 列必填；无默认值</x:v>
+      </x:c>
+      <x:c r="C21" s="61" t="str">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E21" s="61" t="str">
+        <x:v>Required: G PPAP Date, H Technology, I 12 MR Qty, K RFQ Qty Serial.
+I/J/K have no defaults. Optional J is not written to SAP when blank.
+Cost Breakdown: No/blank clears the checkbox; Yes leaves SAP unchanged.</x:v>
+      </x:c>
+      <x:c r="F21" s="61"/>
+      <x:c r="G21" s="61"/>
+      <x:c r="H21" s="61"/>
+    </x:row>
+    <x:row r="22" ht="46" customHeight="1">
+      <x:c r="A22" s="61" t="str">
+        <x:v>RFQ Qty Prototype</x:v>
+      </x:c>
+      <x:c r="B22" s="61" t="str">
+        <x:v>J 列选填；留空不写入 SAP 数量</x:v>
+      </x:c>
+      <x:c r="C22" s="61" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E22" s="61"/>
+      <x:c r="F22" s="61"/>
+      <x:c r="G22" s="61"/>
+      <x:c r="H22" s="61"/>
+    </x:row>
+    <x:row r="23" ht="46" customHeight="1">
+      <x:c r="A23" s="61" t="str">
+        <x:v>RFQ Qty Serial</x:v>
+      </x:c>
+      <x:c r="B23" s="61" t="str">
+        <x:v>K 列必填；无默认值</x:v>
+      </x:c>
+      <x:c r="C23" s="61" t="str">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E23" s="61"/>
+      <x:c r="F23" s="61"/>
+      <x:c r="G23" s="61"/>
+      <x:c r="H23" s="61"/>
+    </x:row>
+    <x:row r="24" ht="46" customHeight="1">
+      <x:c r="A24" s="61" t="str">
+        <x:v>Cost Breakdown</x:v>
+      </x:c>
+      <x:c r="B24" s="61" t="str">
+        <x:v>No / 空白取消勾选；Yes 不操作，保留 SAP 原状态</x:v>
+      </x:c>
+      <x:c r="C24" s="61" t="str">
+        <x:v>No / Yes</x:v>
+      </x:c>
+      <x:c r="E24" s="61"/>
+      <x:c r="F24" s="61"/>
+      <x:c r="G24" s="61"/>
+      <x:c r="H24" s="61"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
     <x:mergeCell ref="A4:H4"/>
     <x:mergeCell ref="A10:H10"/>
+    <x:mergeCell ref="E18:H19"/>
+    <x:mergeCell ref="E21:H24"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>